<commit_message>
chore: update scraped articles with latest data up to July 20
</commit_message>
<xml_diff>
--- a/output/articles_daily.xlsx
+++ b/output/articles_daily.xlsx
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K27"/>
+  <dimension ref="A1:K31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -3454,6 +3454,178 @@
         </is>
       </c>
     </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>18_156771025</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>조달청, AI·로봇 산업 현장에서 'K-공공조달' 추진 방향 모색</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>조달청</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="inlineStr">
+        <is>
+          <t>https://www.korea.kr/briefing/pressReleaseView.do?newsId=156771025&amp;pageIndex=1&amp;repCodeType=&amp;repCode=&amp;startDate=2025-07-20&amp;endDate=2026-07-20&amp;srchWord=인공지능&amp;period=year</t>
+        </is>
+      </c>
+      <c r="F28" s="2" t="inlineStr"/>
+      <c r="G28" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-20T09:39:57.583940+09:00</t>
+        </is>
+      </c>
+      <c r="H28" s="2" t="inlineStr"/>
+      <c r="I28" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J28" s="2" t="inlineStr"/>
+      <c r="K28" s="2" t="inlineStr">
+        <is>
+          <t>정부부처·청·위원회</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>18_156771105</t>
+        </is>
+      </c>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>인공지능·과학기술로 함께 행복한 대체불가 대한민국</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t>과학기술정보통신부</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="E29" s="2" t="inlineStr">
+        <is>
+          <t>https://www.korea.kr/briefing/pressReleaseView.do?newsId=156771105&amp;pageIndex=1&amp;repCodeType=&amp;repCode=&amp;startDate=2025-07-20&amp;endDate=2026-07-20&amp;srchWord=인공지능&amp;period=year</t>
+        </is>
+      </c>
+      <c r="F29" s="2" t="inlineStr"/>
+      <c r="G29" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-20T09:39:57.584030+09:00</t>
+        </is>
+      </c>
+      <c r="H29" s="2" t="inlineStr"/>
+      <c r="I29" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J29" s="2" t="inlineStr"/>
+      <c r="K29" s="2" t="inlineStr">
+        <is>
+          <t>정부부처·청·위원회</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>18_156771051</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>AI 혁신을 뒷받침하고 국민 권익을 증진하는 예방중심 개인정보 보호 실현</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t>개인정보보호위원회</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="E30" s="2" t="inlineStr">
+        <is>
+          <t>https://www.korea.kr/briefing/pressReleaseView.do?newsId=156771051&amp;pageIndex=1&amp;repCodeType=&amp;repCode=&amp;startDate=2025-07-19&amp;endDate=2026-07-19&amp;srchWord=AI&amp;period=year</t>
+        </is>
+      </c>
+      <c r="F30" s="2" t="inlineStr"/>
+      <c r="G30" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-20T09:39:57.584097+09:00</t>
+        </is>
+      </c>
+      <c r="H30" s="2" t="inlineStr"/>
+      <c r="I30" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J30" s="2" t="inlineStr"/>
+      <c r="K30" s="2" t="inlineStr">
+        <is>
+          <t>정부부처·청·위원회</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>18_156771071</t>
+        </is>
+      </c>
+      <c r="B31" s="2" t="inlineStr">
+        <is>
+          <t>AI·과학기술로 함께 행복한 대체불가 대한민국</t>
+        </is>
+      </c>
+      <c r="C31" s="2" t="inlineStr">
+        <is>
+          <t>우주항공청</t>
+        </is>
+      </c>
+      <c r="D31" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="E31" s="2" t="inlineStr">
+        <is>
+          <t>https://www.korea.kr/briefing/pressReleaseView.do?newsId=156771071&amp;pageIndex=1&amp;repCodeType=&amp;repCode=&amp;startDate=2025-07-20&amp;endDate=2026-07-20&amp;srchWord=AI&amp;period=year</t>
+        </is>
+      </c>
+      <c r="F31" s="2" t="inlineStr"/>
+      <c r="G31" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-20T09:39:57.584167+09:00</t>
+        </is>
+      </c>
+      <c r="H31" s="2" t="inlineStr"/>
+      <c r="I31" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J31" s="2" t="inlineStr"/>
+      <c r="K31" s="2" t="inlineStr">
+        <is>
+          <t>정부부처·청·위원회</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:K1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3466,7 +3638,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F5"/>
+  <dimension ref="A1:F11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -3595,6 +3767,138 @@
       </c>
       <c r="F5" t="n">
         <v>63.3</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-07-20T09:39:29.652326+09:00</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>50</v>
+      </c>
+      <c r="C6" t="n">
+        <v>4</v>
+      </c>
+      <c r="D6" t="n">
+        <v>10</v>
+      </c>
+      <c r="E6" t="n">
+        <v>0</v>
+      </c>
+      <c r="F6" t="n">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-07-20T09:40:10.213648+09:00</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>50</v>
+      </c>
+      <c r="C7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D7" t="n">
+        <v>14</v>
+      </c>
+      <c r="E7" t="n">
+        <v>0</v>
+      </c>
+      <c r="F7" t="n">
+        <v>27.1</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-07-20T09:40:37.554731+09:00</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>50</v>
+      </c>
+      <c r="C8" t="n">
+        <v>0</v>
+      </c>
+      <c r="D8" t="n">
+        <v>14</v>
+      </c>
+      <c r="E8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F8" t="n">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-07-20T09:41:05.843776+09:00</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>50</v>
+      </c>
+      <c r="C9" t="n">
+        <v>0</v>
+      </c>
+      <c r="D9" t="n">
+        <v>14</v>
+      </c>
+      <c r="E9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F9" t="n">
+        <v>28.1</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-07-20T09:41:34.251823+09:00</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>50</v>
+      </c>
+      <c r="C10" t="n">
+        <v>0</v>
+      </c>
+      <c r="D10" t="n">
+        <v>14</v>
+      </c>
+      <c r="E10" t="n">
+        <v>0</v>
+      </c>
+      <c r="F10" t="n">
+        <v>28.3</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-07-20T09:42:02.791627+09:00</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>50</v>
+      </c>
+      <c r="C11" t="n">
+        <v>0</v>
+      </c>
+      <c r="D11" t="n">
+        <v>14</v>
+      </c>
+      <c r="E11" t="n">
+        <v>0</v>
+      </c>
+      <c r="F11" t="n">
+        <v>25.9</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
🤖 자동 수집: 2026-07-21 09:04 KST
</commit_message>
<xml_diff>
--- a/output/articles_daily.xlsx
+++ b/output/articles_daily.xlsx
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K31"/>
+  <dimension ref="A1:K35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -3626,6 +3626,432 @@
         </is>
       </c>
     </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>18_156771315</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>"제주공항·한강공원서 '인공지능 윤리' 즐기세요"</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>방송미디어통신위원회</t>
+        </is>
+      </c>
+      <c r="D32" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="E32" s="2" t="inlineStr">
+        <is>
+          <t>https://www.korea.kr/briefing/pressReleaseView.do?newsId=156771315&amp;pageIndex=1&amp;repCodeType=&amp;repCode=&amp;startDate=2025-07-21&amp;endDate=2026-07-21&amp;srchWord=인공지능&amp;period=year</t>
+        </is>
+      </c>
+      <c r="F32" s="2" t="inlineStr">
+        <is>
+          <t>"제주공항·한강공원서 '인공지능 윤리' 즐기세요"
+"제주공항·한강공원서 '인공지능 윤리' 즐기세요"
+- 7월 20~26일 '디지털윤리주간' 운영…전국 각지서 다양한 온·오프라인 행사 -
+제주·김포공항과 여의도 한강공원 등지에서 일상 속 인공지능 윤리를 경험하고 실천해 볼 수 있는 다양한 온·오프라인 행사가 진행된다.
+방송미디어통신위원회(위원장 김종철)와 한국지능정보사회진흥원(원장 김형철)은 7월 20일부터 26일까지 7일간 안전하고 책임있는 인공지능 활용 문화 확산 및 디지털윤리 실천을 위해 '2026년 디지털윤리주간'을 운영한다고 밝혔다.
+올해로 17번째를 맞이하는 디지털윤리주간은 '인공지능과 함께, 윤리도 함께(AI Together, Ethics Together)'를 주제로 가까운 생활공간과 온라인에서 일상 속 인공지능 윤리 관련 다양한 경험을 할 수 있는 참여형 온·오프라인 행사로 진행된다.
+오프라인 행사는 ▲일하는 곳에서 만나는 인공지능 윤리(업무지구) ▲여행길에서 함께하는 인공지능 윤리(관광거점) ▲휴일 일상에서 즐기는 인공지능 윤리(여가공간) ▲학교 현장에서 실천하는 인공지능 윤리(특별교육) 등 4가지 분야로 구성된다.
+광교테크노밸리, 나주혁신도시에서 진행되는 '업무지구' 행사에서는 커피차와 함께 인공지능 윤리 유형찾기, 랜덤 퀴즈뽑기를 통해 일터 속 인공지능 윤리의 현주소를 진단해 보고 올바른 다짐 캠페인을 실천해 본다.
+'관광거점'인 제주공항과 김포공항에서는 '안전한 여행, 안전한 인공지능'이라는 주제로 미션 룰렛과 퀴즈 챌린지를 통해 여행객들에게 인공지능 윤리를 쉽게 배우고 실천하는 경험을 제공할 예정이다.
+여의도 한강공원과 대구 안심도서관 등 '여가공간'에서는 디지털윤리 실천 다짐과 공감 투표를 통해 국민이 스스로 인공지능 활용 원칙을 생각해 보는 기회를 제공한다.
+마지막으로 교장·교감 등 학교 경영자를 대상으로 인공지능 윤리 특별 과정을 운영하여 인공지능 시대의 교육환경 변화와 기술 특성을 이해하고, 학교 내 관련 이슈에 대응할 수 있는 리더십 역량 함양을 지원한다.
+온라인에서도 국민 누구나 쉽게 참여할 수 있는 프로그램을 운영한다.
+디지털윤리 누리집(디지털윤리.kr)에서는 '딥페이크 악용 그만(STOP)!' 빙고 게임을 통해 관련 피해 예방 수칙을 알린다. 또한, 배달앱 '배달의민족'과 함께 디지털윤리 능력 고사를 운영해 퀴즈 참여자에게 할인 쿠폰을 제공할 예정이다.
+방미통위는 전국에서 운영되는 오프라인 캠페인 참여 후기를 작성하거나 개인 사회관계망서비스(SNS)에 인증사진을 게시한 참여자를 대상으로 추첨을 통해 경품을 제공하는 이벤트도 함께 진행한다.
+디지털윤리주간에 대한 보다 자세한 사항은 디지털윤리 누리집(디지털윤리.kr)과 디지털포용 인스타그램(@kdigitalculture)을 통해서도 확인할 수 있다.
+김종철 방미통위원장은 "국민과 함께 인공지능 시대에 필요한 디지털윤리에 대해 공감대를 확산하고 책임있는 디지털 시민의식을 함양하기 위한 행사"라며 "인공지능 윤리를 쉽고 재미있게 배우고 실천할 수 있도록 다양한 교육과 체험프로그램을 계속해서 확대해 나가겠다"고 말했다.
+붙임. '2026년 디지털윤리주간' 안내 전단
+“이 자료는 방송미디어통신위원회의 보도자료를 전재하여 제공함을 알려드립니다.”</t>
+        </is>
+      </c>
+      <c r="G32" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-21T09:03:51.975998+09:00</t>
+        </is>
+      </c>
+      <c r="H32" s="2" t="inlineStr">
+        <is>
+          <t>인공지능, AI, 윤리</t>
+        </is>
+      </c>
+      <c r="I32" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J32" s="2" t="inlineStr">
+        <is>
+          <t>"제주공항·한강공원서 '인공지능 윤리' 즐기세요"
+"제주공항·한강공원서 '인공지능 윤리' 즐기세요"
+- 7월 20~26일 '디지털윤리주간' 운영…전국 각지서 다양한 온·오프라인 행사 -
+제주·김포공항과 여의도 한강공원 등지에서 일상 속 인공지능 윤리를 경험하고 실천해 볼 수 있는 다양한 온·오프라인 행사가 진행된다. 방송미디어통신위원회(위원장 김종철)와 한국지능정보사회진흥원(원장 김형철)은 7월 20일부터 26일까지 7일간 안전하고 책임있는 인공지능 활용 문화 확산 및 디지털윤리 실천을 위해 '2026년 디지털윤리주간'을 운영한다고 밝혔다. 올해로 17번째를 맞이하는 디지털윤리주간은 '인공지능과 함께, 윤리도 함께(AI Together, Ethics Together)'를 주제로 가까운 생활공간과 온라인에서 일상 속 인공지능 윤리 관련 다양한 경험을 할 수 있는 참여형 온·오프라인 행사로 진행된다.</t>
+        </is>
+      </c>
+      <c r="K32" s="2" t="inlineStr">
+        <is>
+          <t>정부부처·청·위원회</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>18_156771398</t>
+        </is>
+      </c>
+      <c r="B33" s="2" t="inlineStr">
+        <is>
+          <t>과기정통부, 「K-문샷 AI 신약 미션」 본격 추진을 위한 현장 소통 나서</t>
+        </is>
+      </c>
+      <c r="C33" s="2" t="inlineStr">
+        <is>
+          <t>과학기술정보통신부</t>
+        </is>
+      </c>
+      <c r="D33" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="E33" s="2" t="inlineStr">
+        <is>
+          <t>https://www.korea.kr/briefing/pressReleaseView.do?newsId=156771398&amp;pageIndex=1&amp;repCodeType=&amp;repCode=&amp;startDate=2025-07-21&amp;endDate=2026-07-21&amp;srchWord=AI&amp;period=year</t>
+        </is>
+      </c>
+      <c r="F33" s="2" t="inlineStr">
+        <is>
+          <t>청와대 소식
+공직메일
+알림설정OFF
+상세검색
+과기정통부, 「K-문샷 AI 신약 미션」 본격 추진을 위한 현장 소통 나서
+2026.07.20 과학기술정보통신부
+첨부파일
+260721 조간 (보도) K-문샷 AI 신약 미션 현장의견 수렴회 개최.hwpx
+260721 조간 (보도) K-문샷 AI 신약 미션 현장의견 수렴회 개최.odt
+“이 자료는 과학기술정보통신부의 보도자료를 전재하여 제공함을 알려드립니다.”
+인류의 유산, 세계의 약속
+정부-홈쇼핑-중소기업, 상생협력 약속
+"화장실 갈 시간도 없어요" 국민신문고 민원 처리하는 공정위 직원의 REAL 하루
+당뇨병전단계 성인을 위한 식사지침
+국내 첫 세계유산위원회 부산 개막…대한민국 주도 '부산 선언' 채택
+맞벌이 주목! 초등방학 '틈새돌봄'으로 점심·저녁 제공
+경찰관 가족 사건 상피제 도입…'제식구 감싸기' 근절
+공무원이 직접 만든 AI 법령 비서 시범 개시
+저소득층에 더 큰 힘으로 다가온 '두 차례의 민생 지원금'
+정부, 550조 AI 데이터센터 투자 견인…'1인 1 AI 에이전트' 시대 연다
+하반기 3% 이내 물가관리 총력…3대 메가프로젝트 역량 집중
+이 대통령 "잠재성장률 3%·세계무역 4강·국민소득 5만불 원년으로"
+잠재성장률 3%·수출 4강·국민소득 5만 달러…'경제 대도약 원년'
+최신뉴스
+국민신문고 민원 처리하는 공정위 직원의 REAL 하루
+2026년 하반기 온누리상품권, 이렇게 달라집니다!
+불법 사교육 근절, 신고포상금 10배 인상!
+제48차 유네스코 세계유산위원회 개회식
+정책포커스
+산업통상부 (설명자료)유통상생 기금 등 상생방안에 관해 구체적으로 논의하거나 확정된 사항은 없습니다 2026.07.21
+산업통상부 (설명자료)유통상생 기금 등 상생방안에 관해 구체적으로 논의하거나 확정된 사항은 없습니다 2026.07.21
+정책브리핑 RSS 서비스 제공 중단 안내
+(30119) 세종특별자치시 갈매로 388 정부세종청사 15동 © 문화체육관광부
+X 바로가기
+네이버포스트 바로가기
+유튜브 바로가기
+인스타그램 바로가기
+행정부처 바로가기</t>
+        </is>
+      </c>
+      <c r="G33" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-21T09:04:01.620481+09:00</t>
+        </is>
+      </c>
+      <c r="H33" s="2" t="inlineStr">
+        <is>
+          <t>AI, 데이터</t>
+        </is>
+      </c>
+      <c r="I33" s="2" t="n">
+        <v>0.613</v>
+      </c>
+      <c r="J33" s="2" t="inlineStr">
+        <is>
+          <t>청와대 소식
+공직메일
+알림설정OFF
+상세검색
+과기정통부, 「K-문샷 AI 신약 미션」 본격 추진을 위한 현장 소통 나서
+2026.07.20 과학기술정보통신부
+첨부파일
+260721 조간 (보도) K-문샷 AI 신약 미션 현장의견 수렴회 개최.hwpx
+260721 조간 (보도) K-문샷 AI 신약 미션 현장의견 수렴회 개최.odt
+“이 자료는 과학기술정보통신부의 보도자료를 전재하여 제공함을 알려드립니다.”
+인류의 유산, 세계의 약속
+정부-홈쇼핑-중소기업, 상생협력 약속
+"화장실 갈 시간도 없어요" 국민신문고 민원 처리하는 공정위 직원의 REAL 하루
+당뇨병전단계 성인을 위한 식사지침
+국내 첫 세계유산위원회 부산 개막…대한민국 주도 '부산 선언' 채택
+맞벌이 주목! 초등방학 '틈새돌봄'으로 점심·저녁 제공
+경찰관 가족 사건 상피제 도입…'제식구 감싸기' 근절
+공무원이 직접 만든 AI 법령 비서 시범 개시
+저소득층에 더 큰 힘으로 다가온 '두 차례의 민생 지원금'
+정부, 550조 AI 데이터센터 투자 견인…'1인 1 AI 에이전트' 시대 연다
+하반기 3% 이내 물가관리 총력…3대 메가프로젝트 역량 집중
+이 대통령 "잠재성장률 3%·세계무역 4강·국민소득 5만불 원년으로"
+잠재성장률 3%·수출 4강·국민소득 5만 달러…'경제 대도약 원년'
+최신뉴스
+국민신문고 민원 처리하는 공정위 직원의 REAL 하루
+2026년 하반기 온누리상품권, 이렇게 달라집니다! 불법 사교육 근절, 신고포상금 10배 인상!</t>
+        </is>
+      </c>
+      <c r="K33" s="2" t="inlineStr">
+        <is>
+          <t>정부부처·청·위원회</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>18_156771410</t>
+        </is>
+      </c>
+      <c r="B34" s="2" t="inlineStr">
+        <is>
+          <t>인공지능(AI) 및 안전보건 분야 업무교류로 감사역량 강화한다</t>
+        </is>
+      </c>
+      <c r="C34" s="2" t="inlineStr">
+        <is>
+          <t>고용노동부</t>
+        </is>
+      </c>
+      <c r="D34" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="E34" s="2" t="inlineStr">
+        <is>
+          <t>https://www.korea.kr/briefing/pressReleaseView.do?newsId=156771410&amp;pageIndex=1&amp;repCodeType=&amp;repCode=&amp;startDate=2025-07-21&amp;endDate=2026-07-21&amp;srchWord=인공지능&amp;period=year</t>
+        </is>
+      </c>
+      <c r="F34" s="2" t="inlineStr">
+        <is>
+          <t>청와대 소식
+공직메일
+알림설정OFF
+상세검색
+인공지능(AI) 및 안전보건 분야 업무교류로 감사역량 강화한다
+2026.07.20 고용노동부
+첨부파일
+260720_보도자료_안전보건공단-한국수자원공사 자체감사기구 업무협약(안전보건공단).pdf
+260720_보도자료_안전보건공단-한국수자원공사 자체감사기구 업무협약(안전보건공단).hwpx
+“이 자료는 고용노동부의 보도자료를 전재하여 제공함을 알려드립니다.”
+"청년의 취업성공 경험이 미래를 바꾼다" 「청년미래플러스」 열린 소통 간담회 개최
+(참고자료)유미진 주제네바 대표부 1등 서기관 세계무역기구(WTO) 수입허가 위원회 의장으로 선출
+"화장실 갈 시간도 없어요" 국민신문고 민원 처리하는 공정위 직원의 REAL 하루
+당뇨병전단계 성인을 위한 식사지침
+국내 첫 세계유산위원회 부산 개막…대한민국 주도 '부산 선언' 채택
+맞벌이 주목! 초등방학 '틈새돌봄'으로 점심·저녁 제공
+경찰관 가족 사건 상피제 도입…'제식구 감싸기' 근절
+공무원이 직접 만든 AI 법령 비서 시범 개시
+저소득층에 더 큰 힘으로 다가온 '두 차례의 민생 지원금'
+정부, 550조 AI 데이터센터 투자 견인…'1인 1 AI 에이전트' 시대 연다
+하반기 3% 이내 물가관리 총력…3대 메가프로젝트 역량 집중
+이 대통령 "잠재성장률 3%·세계무역 4강·국민소득 5만불 원년으로"
+잠재성장률 3%·수출 4강·국민소득 5만 달러…'경제 대도약 원년'
+최신뉴스
+국민신문고 민원 처리하는 공정위 직원의 REAL 하루
+2026년 하반기 온누리상품권, 이렇게 달라집니다!
+불법 사교육 근절, 신고포상금 10배 인상!
+제48차 유네스코 세계유산위원회 개회식
+정책포커스
+산업통상부 (설명자료)유통상생 기금 등 상생방안에 관해 구체적으로 논의하거나 확정된 사항은 없습니다 2026.07.21
+산업통상부 (설명자료)유통상생 기금 등 상생방안에 관해 구체적으로 논의하거나 확정된 사항은 없습니다 2026.07.21
+정책브리핑 RSS 서비스 제공 중단 안내
+(30119) 세종특별자치시 갈매로 388 정부세종청사 15동 © 문화체육관광부
+X 바로가기
+네이버포스트 바로가기
+유튜브 바로가기
+인스타그램 바로가기
+행정부처 바로가기</t>
+        </is>
+      </c>
+      <c r="G34" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-21T09:04:09.911741+09:00</t>
+        </is>
+      </c>
+      <c r="H34" s="2" t="inlineStr">
+        <is>
+          <t>AI, 인공지능, 데이터</t>
+        </is>
+      </c>
+      <c r="I34" s="2" t="n">
+        <v>0.531</v>
+      </c>
+      <c r="J34" s="2" t="inlineStr">
+        <is>
+          <t>청와대 소식
+공직메일
+알림설정OFF
+상세검색
+인공지능(AI) 및 안전보건 분야 업무교류로 감사역량 강화한다
+2026.07.20 고용노동부
+첨부파일
+260720_보도자료_안전보건공단-한국수자원공사 자체감사기구 업무협약(안전보건공단).pdf
+260720_보도자료_안전보건공단-한국수자원공사 자체감사기구 업무협약(안전보건공단).hwpx
+“이 자료는 고용노동부의 보도자료를 전재하여 제공함을 알려드립니다.”
+"청년의 취업성공 경험이 미래를 바꾼다" 「청년미래플러스」 열린 소통 간담회 개최
+(참고자료)유미진 주제네바 대표부 1등 서기관 세계무역기구(WTO) 수입허가 위원회 의장으로 선출
+"화장실 갈 시간도 없어요" 국민신문고 민원 처리하는 공정위 직원의 REAL 하루
+당뇨병전단계 성인을 위한 식사지침
+국내 첫 세계유산위원회 부산 개막…대한민국 주도 '부산 선언' 채택
+맞벌이 주목! 초등방학 '틈새돌봄'으로 점심·저녁 제공
+경찰관 가족 사건 상피제 도입…'제식구 감싸기' 근절
+공무원이 직접 만든 AI 법령 비서 시범 개시
+저소득층에 더 큰 힘으로 다가온 '두 차례의 민생 지원금'
+정부, 550조 AI 데이터센터 투자 견인…'1인 1 AI 에이전트' 시대 연다
+하반기 3% 이내 물가관리 총력…3대 메가프로젝트 역량 집중
+이 대통령 "잠재성장률 3%·세계무역 4강·국민소득 5만불 원년으로"
+잠재성장률 3%·수출 4강·국민소득 5만 달러…'경제 대도약 원년'
+최신뉴스
+국민신문고 민원 처리하는 공정위 직원의 REAL 하루
+2026년 하반기 온누리상품권, 이렇게 달라집니다! 불법 사교육 근절, 신고포상금 10배 인상!</t>
+        </is>
+      </c>
+      <c r="K34" s="2" t="inlineStr">
+        <is>
+          <t>정부부처·청·위원회</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>18_156771346</t>
+        </is>
+      </c>
+      <c r="B35" s="2" t="inlineStr">
+        <is>
+          <t>다양한 소재부품 공정을 하나의 M.AX로, 반월시화에서 시작되는 '중소의 기적'</t>
+        </is>
+      </c>
+      <c r="C35" s="2" t="inlineStr">
+        <is>
+          <t>산업통상부</t>
+        </is>
+      </c>
+      <c r="D35" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="E35" s="2" t="inlineStr">
+        <is>
+          <t>https://www.korea.kr/briefing/pressReleaseView.do?newsId=156771346&amp;pageIndex=1&amp;repCodeType=&amp;repCode=&amp;startDate=2025-07-21&amp;endDate=2026-07-21&amp;srchWord=AI&amp;period=year</t>
+        </is>
+      </c>
+      <c r="F35" s="2" t="inlineStr">
+        <is>
+          <t>청와대 소식
+공직메일
+알림설정OFF
+상세검색
+다양한 소재부품 공정을 하나의 M.AX로, 반월시화에서 시작되는 '중소의 기적'
+2026.07.20 산업통상부
+첨부파일
+0717(20석간, 20일(월) 09시엠바고)입지총괄과, 반월시화 소부장 MINI 얼라이언스 간담회.pdf
+0717(20석간, 20일(월) 09시엠바고)입지총괄과, 반월시화 소부장 MINI 얼라이언스 간담회.hwpx
+“이 자료는 산업통상부의 보도자료를 전재하여 제공함을 알려드립니다.”
+기업 지방투자 촉진을 위해 지방투자촉진보조금 지원기준 개선
+농식품부, K-농기자재 해외시장 개척 속도 낸다 2026년 바이어초청 수출상담회(K-AgroEX) 개최
+"화장실 갈 시간도 없어요" 국민신문고 민원 처리하는 공정위 직원의 REAL 하루
+당뇨병전단계 성인을 위한 식사지침
+국내 첫 세계유산위원회 부산 개막…대한민국 주도 '부산 선언' 채택
+맞벌이 주목! 초등방학 '틈새돌봄'으로 점심·저녁 제공
+경찰관 가족 사건 상피제 도입…'제식구 감싸기' 근절
+공무원이 직접 만든 AI 법령 비서 시범 개시
+저소득층에 더 큰 힘으로 다가온 '두 차례의 민생 지원금'
+정부, 550조 AI 데이터센터 투자 견인…'1인 1 AI 에이전트' 시대 연다
+하반기 3% 이내 물가관리 총력…3대 메가프로젝트 역량 집중
+이 대통령 "잠재성장률 3%·세계무역 4강·국민소득 5만불 원년으로"
+잠재성장률 3%·수출 4강·국민소득 5만 달러…'경제 대도약 원년'
+최신뉴스
+국민신문고 민원 처리하는 공정위 직원의 REAL 하루
+2026년 하반기 온누리상품권, 이렇게 달라집니다!
+불법 사교육 근절, 신고포상금 10배 인상!
+제48차 유네스코 세계유산위원회 개회식
+정책포커스
+산업통상부 (설명자료)유통상생 기금 등 상생방안에 관해 구체적으로 논의하거나 확정된 사항은 없습니다 2026.07.21
+산업통상부 (설명자료)유통상생 기금 등 상생방안에 관해 구체적으로 논의하거나 확정된 사항은 없습니다 2026.07.21
+정책브리핑 RSS 서비스 제공 중단 안내
+(30119) 세종특별자치시 갈매로 388 정부세종청사 15동 © 문화체육관광부
+X 바로가기
+네이버포스트 바로가기
+유튜브 바로가기
+인스타그램 바로가기
+행정부처 바로가기</t>
+        </is>
+      </c>
+      <c r="G35" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-21T09:04:17.250844+09:00</t>
+        </is>
+      </c>
+      <c r="H35" s="2" t="inlineStr">
+        <is>
+          <t>AI, AX, 데이터</t>
+        </is>
+      </c>
+      <c r="I35" s="2" t="n">
+        <v>0.417</v>
+      </c>
+      <c r="J35" s="2" t="inlineStr">
+        <is>
+          <t>청와대 소식
+공직메일
+알림설정OFF
+상세검색
+다양한 소재부품 공정을 하나의 M.AX로, 반월시화에서 시작되는 '중소의 기적'
+2026.07.20 산업통상부
+첨부파일
+0717(20석간, 20일(월) 09시엠바고)입지총괄과, 반월시화 소부장 MINI 얼라이언스 간담회.pdf
+0717(20석간, 20일(월) 09시엠바고)입지총괄과, 반월시화 소부장 MINI 얼라이언스 간담회.hwpx
+“이 자료는 산업통상부의 보도자료를 전재하여 제공함을 알려드립니다.”
+기업 지방투자 촉진을 위해 지방투자촉진보조금 지원기준 개선
+농식품부, K-농기자재 해외시장 개척 속도 낸다 2026년 바이어초청 수출상담회(K-AgroEX) 개최
+"화장실 갈 시간도 없어요" 국민신문고 민원 처리하는 공정위 직원의 REAL 하루
+당뇨병전단계 성인을 위한 식사지침
+국내 첫 세계유산위원회 부산 개막…대한민국 주도 '부산 선언' 채택
+맞벌이 주목! 초등방학 '틈새돌봄'으로 점심·저녁 제공
+경찰관 가족 사건 상피제 도입…'제식구 감싸기' 근절
+공무원이 직접 만든 AI 법령 비서 시범 개시
+저소득층에 더 큰 힘으로 다가온 '두 차례의 민생 지원금'
+정부, 550조 AI 데이터센터 투자 견인…'1인 1 AI 에이전트' 시대 연다
+하반기 3% 이내 물가관리 총력…3대 메가프로젝트 역량 집중
+이 대통령 "잠재성장률 3%·세계무역 4강·국민소득 5만불 원년으로"
+잠재성장률 3%·수출 4강·국민소득 5만 달러…'경제 대도약 원년'
+최신뉴스
+국민신문고 민원 처리하는 공정위 직원의 REAL 하루
+2026년 하반기 온누리상품권, 이렇게 달라집니다! 불법 사교육 근절, 신고포상금 10배 인상!</t>
+        </is>
+      </c>
+      <c r="K35" s="2" t="inlineStr">
+        <is>
+          <t>정부부처·청·위원회</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:K1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3638,7 +4064,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F11"/>
+  <dimension ref="A1:F12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -3899,6 +4325,28 @@
       </c>
       <c r="F11" t="n">
         <v>25.9</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2026-07-21T09:03:36.463574+09:00</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>50</v>
+      </c>
+      <c r="C12" t="n">
+        <v>4</v>
+      </c>
+      <c r="D12" t="n">
+        <v>5</v>
+      </c>
+      <c r="E12" t="n">
+        <v>0</v>
+      </c>
+      <c r="F12" t="n">
+        <v>58.9</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
🤖 자동 수집: 2026-07-21 10:57 KST
</commit_message>
<xml_diff>
--- a/output/articles_daily.xlsx
+++ b/output/articles_daily.xlsx
@@ -4064,7 +4064,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F12"/>
+  <dimension ref="A1:F13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -4347,6 +4347,28 @@
       </c>
       <c r="F12" t="n">
         <v>58.9</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2026-07-21T10:56:38.424455+09:00</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>50</v>
+      </c>
+      <c r="C13" t="n">
+        <v>0</v>
+      </c>
+      <c r="D13" t="n">
+        <v>10</v>
+      </c>
+      <c r="E13" t="n">
+        <v>0</v>
+      </c>
+      <c r="F13" t="n">
+        <v>35.8</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
🤖 자동 수집: 2026-07-21 11:10 KST
</commit_message>
<xml_diff>
--- a/output/articles_daily.xlsx
+++ b/output/articles_daily.xlsx
@@ -4064,7 +4064,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F13"/>
+  <dimension ref="A1:F14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -4369,6 +4369,28 @@
       </c>
       <c r="F13" t="n">
         <v>35.8</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-07-21T11:09:51.653170+09:00</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>50</v>
+      </c>
+      <c r="C14" t="n">
+        <v>0</v>
+      </c>
+      <c r="D14" t="n">
+        <v>10</v>
+      </c>
+      <c r="E14" t="n">
+        <v>0</v>
+      </c>
+      <c r="F14" t="n">
+        <v>35.9</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
🤖 자동 수집: 2026-07-21 11:26 KST
</commit_message>
<xml_diff>
--- a/output/articles_daily.xlsx
+++ b/output/articles_daily.xlsx
@@ -4064,7 +4064,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F14"/>
+  <dimension ref="A1:F15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -4391,6 +4391,28 @@
       </c>
       <c r="F14" t="n">
         <v>35.9</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2026-07-21T11:25:46.315776+09:00</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>50</v>
+      </c>
+      <c r="C15" t="n">
+        <v>0</v>
+      </c>
+      <c r="D15" t="n">
+        <v>10</v>
+      </c>
+      <c r="E15" t="n">
+        <v>0</v>
+      </c>
+      <c r="F15" t="n">
+        <v>34.3</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
🤖 자동 수집: 2026-07-21 13:36 KST
</commit_message>
<xml_diff>
--- a/output/articles_daily.xlsx
+++ b/output/articles_daily.xlsx
@@ -4462,7 +4462,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F16"/>
+  <dimension ref="A1:F17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -4833,6 +4833,28 @@
       </c>
       <c r="F16" t="n">
         <v>62.6</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2026-07-21T13:36:27.456997+09:00</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>50</v>
+      </c>
+      <c r="C17" t="n">
+        <v>0</v>
+      </c>
+      <c r="D17" t="n">
+        <v>11</v>
+      </c>
+      <c r="E17" t="n">
+        <v>0</v>
+      </c>
+      <c r="F17" t="n">
+        <v>16.2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
🤖 자동 수집: 2026-07-21 13:39 KST
</commit_message>
<xml_diff>
--- a/output/articles_daily.xlsx
+++ b/output/articles_daily.xlsx
@@ -4462,7 +4462,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F17"/>
+  <dimension ref="A1:F18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -4854,6 +4854,28 @@
         <v>0</v>
       </c>
       <c r="F17" t="n">
+        <v>16.2</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>2026-07-21T13:39:16.833686+09:00</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>50</v>
+      </c>
+      <c r="C18" t="n">
+        <v>0</v>
+      </c>
+      <c r="D18" t="n">
+        <v>11</v>
+      </c>
+      <c r="E18" t="n">
+        <v>0</v>
+      </c>
+      <c r="F18" t="n">
         <v>16.2</v>
       </c>
     </row>

</xml_diff>

<commit_message>
🤖 자동 수집: 2026-07-21 13:42 KST
</commit_message>
<xml_diff>
--- a/output/articles_daily.xlsx
+++ b/output/articles_daily.xlsx
@@ -4462,7 +4462,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F18"/>
+  <dimension ref="A1:F19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -4877,6 +4877,28 @@
       </c>
       <c r="F18" t="n">
         <v>16.2</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>2026-07-21T13:42:32.370783+09:00</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>50</v>
+      </c>
+      <c r="C19" t="n">
+        <v>0</v>
+      </c>
+      <c r="D19" t="n">
+        <v>11</v>
+      </c>
+      <c r="E19" t="n">
+        <v>0</v>
+      </c>
+      <c r="F19" t="n">
+        <v>16.7</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
🤖 자동 수집: 2026-07-21 13:48 KST
</commit_message>
<xml_diff>
--- a/output/articles_daily.xlsx
+++ b/output/articles_daily.xlsx
@@ -4462,7 +4462,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F19"/>
+  <dimension ref="A1:F20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -4899,6 +4899,28 @@
       </c>
       <c r="F19" t="n">
         <v>16.7</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>2026-07-21T13:48:37.421499+09:00</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>50</v>
+      </c>
+      <c r="C20" t="n">
+        <v>0</v>
+      </c>
+      <c r="D20" t="n">
+        <v>11</v>
+      </c>
+      <c r="E20" t="n">
+        <v>0</v>
+      </c>
+      <c r="F20" t="n">
+        <v>15.6</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
🤖 자동 수집: 2026-07-21 13:52 KST
</commit_message>
<xml_diff>
--- a/output/articles_daily.xlsx
+++ b/output/articles_daily.xlsx
@@ -4462,7 +4462,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F20"/>
+  <dimension ref="A1:F21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -4920,6 +4920,28 @@
         <v>0</v>
       </c>
       <c r="F20" t="n">
+        <v>15.6</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>2026-07-21T13:52:32.045975+09:00</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>50</v>
+      </c>
+      <c r="C21" t="n">
+        <v>0</v>
+      </c>
+      <c r="D21" t="n">
+        <v>11</v>
+      </c>
+      <c r="E21" t="n">
+        <v>0</v>
+      </c>
+      <c r="F21" t="n">
         <v>15.6</v>
       </c>
     </row>

</xml_diff>

<commit_message>
🤖 자동 수집: 2026-07-21 14:08 KST
</commit_message>
<xml_diff>
--- a/output/articles_daily.xlsx
+++ b/output/articles_daily.xlsx
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K36"/>
+  <dimension ref="A1:K37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -4450,6 +4450,148 @@
         </is>
       </c>
     </row>
+    <row r="37">
+      <c r="A37" s="2" t="inlineStr">
+        <is>
+          <t>1_461449</t>
+        </is>
+      </c>
+      <c r="B37" s="2" t="inlineStr">
+        <is>
+          <t>AI 환각(할루시네이션 현상) 줄인다. 서울시, 공공데이터 최초 MCP 서비스 개시</t>
+        </is>
+      </c>
+      <c r="C37" s="2" t="inlineStr">
+        <is>
+          <t>서울특별시</t>
+        </is>
+      </c>
+      <c r="D37" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-12</t>
+        </is>
+      </c>
+      <c r="E37" s="2" t="inlineStr">
+        <is>
+          <t>https://www.seoul.go.kr/news/news_report.do#view/461449</t>
+        </is>
+      </c>
+      <c r="F37" s="2" t="inlineStr">
+        <is>
+          <t>HOME
+서울소식
+보도·해명자료
+본문 글자 크기 크게 변경
+본문 글자 크기 작게 변경
+AI 환각(할루시네이션 현상) 줄인다. 서울시, 공공데이터 최초 MCP 서비스 개시
+디지털도시국 데이터전략과
+등록일
+2026-07-12
+수정일
+첨부파일
+바로듣기
+첨부파일
+AI 환각(할루시네이션 현상) 줄인다. 서울시, 공공데이터 최초 MCP 서비스 개시.hwp
+(908 KB Bytes, 다운로드: 308 회 )
+AI 환각(할루시네이션 현상) 줄인다. 서울시, 공공데이터 최초 MCP 서비스 개시
+- 서울 실시간 공공데이터를 AI 개발 환경에서 정확하게 활용하도록 지원
+- 공공데이터 최초 '서울 실시간 도시데이터 MCP' 7월 14일 오전 11시 공개
+- AI 기반 관광·상권 분석 등 에이전트 서비스 활성화 기대
+앞으로 인공지능
+(AI)
+지금 명동은 얼마나 붐비나요
+?", "
+오늘 한강에 가도 될까요
+?", "
+오늘 서울에서 열리는 축제는 무엇인가요
+라고 물으면 인터넷에 떠도는 오래된 정보가 아니라 서울시의 실시간 공공데이터를 바탕으로 답을 받을 수 있게 된다
+서울시는 이러한 서비스를 가능하게 하는
+MCP(Model Context Protocol·
+델 컨텍스트 프로토콜
+를 공공데이터 서비스 최초로 시범 운영한다고 밝혔다
+○ MCP는 AI와 공공데이터를 직접 연결해 주는 기술이다. 지금까지 AI는 학습된 정보나 인터넷 검색 결과를 바탕으로 답을 만들어 잘못된 정보를 사실처럼 말하는 '환각(Hallucination)' 현상이 발생하기도 했다.
+○ 하지만 MCP를 활용하면 AI가 서울시의 최신 공공데이터를 직접 확인한 뒤 답하기 때문에 더욱 정확하고 신뢰할 수 있는 정보를 제공할 수 있다.
+○ MCP는 24년 11월 AI 기업 앤트로픽(Anthropic)이 공개한 기술로, 현재 OpenAI, Google, Kakao 등 세계 주요 AI 기업들도 활용하고 있는 AI 표준 기술이다.
+이번에 제공되는 데이터는 서울시의 대표 공공데이터인
+서울 실시간 도시데이터
+○ 서울 주요 121개 지역의 인구 혼잡도, 대중교통, 날씨, 문화행사 등 다양한 정보를 실시간으로 제공한다.
+○ 지난해 API 조회 건수는 3억2천만 건에 달했으며, 데이터는 수초에서 최대 5분 간격으로 계속 갱신된다.
+○ 서울시는 기존 공공데이터 API를 MCP 방식으로 확장해 AI 에이전트에서도 쉽게 활용할 수 있도록 했다. 이번 개발에는 AI 전문기업 화이트스캔이 참여했다.
+시범서비스는 선착순
+100
+명을 대상으로 운영된다
+○ 이용자는 카카오의 MCP 플랫폼인 PlayMCP를 통해 서비스를 이용할 수 있으며, 신청자에게는 MCP 인증키와 이용 가이드가 제공된다.
+○ 인증키 신청 페이지는 7월 14일 오전 11시에 공개될 예정이다.
+○ 서울시는 시범 운영 후 이용자 의견을 수렴해 서비스 만족도와 활용성을 평가하고, 공공데이터 MCP 서비스 확대 여부를 검토할 계획이다.
+서울시는 이번 서비스를 통해
+가 서울의 실시간 데이터를 활용해
+실시간 관광코스 추천
+혼잡도 안내
+상권 분석
+행사 정보 안내 등 다양한
+서비스를 더욱 정확하게 제공할 수 있을 것으로 기대하고 있다
+정영준
+서울시 디지털도시국장은
+"AI
+시대에는 정확한 데이터가 경쟁력
+이라며
+서울의 공공데이터를 누구나
+에서 쉽고 정확하게 활용할 수 있는 환경을 만들어 가겠다
+고 말했다
+본 저작물은 "공공누리"
+제4유형:출처표시+상업적 이용금지+변경금지
+조건에 따라 이용 할 수 있습니다.
+글퍼가기
+페이지 만족도 조사
+이 페이지에서 제공하는 정보에 대하여 만족하십니까?
+아니오
+5점 - 매우만족
+4점 - 만족
+3점 - 보통
+2점 - 불만족
+1점 - 매우 불만족
+평가하기</t>
+        </is>
+      </c>
+      <c r="G37" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-21T14:08:05.318550+09:00</t>
+        </is>
+      </c>
+      <c r="H37" s="2" t="inlineStr">
+        <is>
+          <t>AI, MCP, 인공지능, 데이터, 플랫폼</t>
+        </is>
+      </c>
+      <c r="I37" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J37" s="2" t="inlineStr">
+        <is>
+          <t>HOME
+서울소식
+보도·해명자료
+본문 글자 크기 크게 변경
+본문 글자 크기 작게 변경
+AI 환각(할루시네이션 현상) 줄인다. 서울시, 공공데이터 최초 MCP 서비스 개시
+디지털도시국 데이터전략과
+등록일
+2026-07-12
+수정일
+첨부파일
+바로듣기
+첨부파일
+AI 환각(할루시네이션 현상) 줄인다. 서울시, 공공데이터 최초 MCP 서비스 개시.hwp
+(908 KB Bytes, 다운로드: 308 회 )
+AI 환각(할루시네이션 현상) 줄인다.</t>
+        </is>
+      </c>
+      <c r="K37" s="2" t="inlineStr">
+        <is>
+          <t>정부부처·청·위원회</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:K1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -4462,7 +4604,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F21"/>
+  <dimension ref="A1:F22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -4943,6 +5085,28 @@
       </c>
       <c r="F21" t="n">
         <v>15.6</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>2026-07-21T14:07:30.425056+09:00</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>7</v>
+      </c>
+      <c r="C22" t="n">
+        <v>1</v>
+      </c>
+      <c r="D22" t="n">
+        <v>0</v>
+      </c>
+      <c r="E22" t="n">
+        <v>0</v>
+      </c>
+      <c r="F22" t="n">
+        <v>65</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
🤖 자동 수집: 2026-07-21 15:19 KST
</commit_message>
<xml_diff>
--- a/output/articles_daily.xlsx
+++ b/output/articles_daily.xlsx
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K39"/>
+  <dimension ref="A1:K45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -4869,6 +4869,1278 @@
         </is>
       </c>
     </row>
+    <row r="40">
+      <c r="A40" s="2" t="inlineStr">
+        <is>
+          <t>15_B000000157512Bc4nI9i</t>
+        </is>
+      </c>
+      <c r="B40" s="2" t="inlineStr">
+        <is>
+          <t>'핵테온 세종' AI·사이버보안 협력 중심지로 자리매김</t>
+        </is>
+      </c>
+      <c r="C40" s="2" t="inlineStr">
+        <is>
+          <t>세종특별자치시</t>
+        </is>
+      </c>
+      <c r="D40" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="E40" s="2" t="inlineStr">
+        <is>
+          <t>https://www.sejong.go.kr/bbs/R0079/view.do?nttId=B000000157512Bc4nI9i&amp;mno=sub02_0401&amp;cmsNoStr=&amp;pageIndex=1&amp;kind=</t>
+        </is>
+      </c>
+      <c r="F40" s="2" t="inlineStr">
+        <is>
+          <t>대메뉴 바로가기
+민원·소통·참여
+여행정보
+세종소개
+정보공개
+분야별정보
+생활정보
+로그인
+회원가입
+SNS
+Languages
+세종특별자치시 세종소개
+전체메뉴
+세종소개
+세종소식
+부서바로가기
+세종소식
+시정소식
+고시/공고
+언론보도자료
+해명자료
+영상자료
+세종사진관
+언론보도자료
+HOME
+세종소식
+언론보도자료
+공유 프린트 짧은URL즐겨찾기
+'핵테온 세종' AI·사이버보안 협력 중심지로 자리매김
+작성자인공지능디지털담당관  조회수138
+등록일2026-07-10
+아이콘
+2026_핵테온_세종(인공지능디지털담당관).JPG [1,706.6 KB]
+아이콘
+2026_핵테온_세종2(인공지능디지털담당관).JPG [1,650.5 KB]
+아이콘
+국제_대학생_사이버보안_경진대회(인공지능디지털담당관).JPG [1,958.9 KB]
+한글 아이콘
+추가260710_핵테온세종(인공지능디지털담당관).HWP [242.8 KB] 추가260710_핵테온세종(인공지능디지털담당관).hwp바로보기
+'핵테온 세종' AI·사이버보안 협력 중심지로 자리매김
+- 국가정보원 공동주최로 위상 강화…47개국 5,000여 명 참여 -
+인재 양성·기술 교류·정책 협력 아우른 융합 플랫폼으로 안착 -
+전 세계 사이버보안 인재와 인공지능 보안 기술·정책 역량이 한 데 모인 ‘2026 핵테온 세종’이 이틀간의 대장정을 성공적으로 마쳤다.
+세종특별자치시(시장 조상호)는 지난 9∼10일 정부세종컨벤션센터에서 국가정보원과 공동으로 ‘2026 핵테온 세종’을 개최했다.
+올해 5회째를 맞은 이번 행사는 국가 차원의 사이버안보 협력 행사로 의미를 더한 가운데 국내외 보안 전문가와 대학생, 기업 관계자 등 5,000여 명이 참여해 인공지능 시대 사이버보안의 해법을 모색했다.
+특히 지능화되는 사이버 위협에 대응할 미래 보안 인재를 발굴·육성하고, 기술·정책·산업 간 협력 기반을 넓히는 자리로 마련됐다.
+우선 글로벌 사이버보안 인재 양성의 등용문인 경진 대회에는 역대 가장 많은 47개국 216개 대학, 548팀 1,799명이 예선에 참가했다.
+본선에 진출한 40개 팀은 총상금 3,800만 원을 두고 치열한 경연을 펼쳤다.
+그 결과 고급 부문 대상은 대한민국 ‘정현수의전역을축하합니다’ 팀이, 초급 부문 대상은 베트남 ‘CyberCh1ck’ 팀이 차지했다.
+경진대회 종료 후에는 대회 참가 학생에게 세종시를 홍보하고, 학생 간 관심 분야 공유 및 친목을 도모하는 교류의 장을 마련했다.
+학술대회에서는 인공지능과 사이버보안 등 관련 기술과 정책, 산업생태계를 아우르는 활발한 논의를 펼쳤다.
+우선 손기욱 한국사이버안보학회장이 ‘AI와 사이버안보, 우리는?’을 주제로 한 강연에서 인공지능 시대 속 미래사회의 대응책을 집중적으로 설명했다.
+이어 야마시타 아키마사 전(前) 교토부 부지사가 지역·현장을 중심으로 인공지능과 사이버보안의 국제협력 방안을 제시했다.
+또한, 국가정보원은 국내 사이버보안 취약점 신고·조치 공개 제도와 인공지능 보완 정책 등 정부 차원의 보완관리 대응 전략을 소개했다.
+42여 개 기업과 기관이 참가한 정보통신기술 전시회와 정보보호학회 우주·양자보안연구회, 과학기술정보보호협의회, 국가사이버안보세미나, 제2회 지방정부 정보보안 실무 협의회 등에서는 공공·민간·학계의 사이버보안 협력 기반을 한층 넓혔다.
+이어 지난달 열린 제2회 초중고교 AI·사이버보안 한마당에서 우수한 성적을 거둔 학생 6명에게 세종시장상과 시교육감상을 수여하면서 사이버보안 미래 인재의 성장을 독려했다.
+시는 핵테온 세종을 계기로 구축한 국가정보원 등 중앙부처, 산·학·연 관계기관과의 협력체계를 바탕으로 교육발전특구와 충청권 정보보호 클러스터 등 핵심 사업을 추진하고 사이버보안 인재 양성에도 힘쓸 방침이다.
+조상호 시장은 “국가균형성장의 중심인 세종에서 열린 핵테온 세종은 대한민국의 디지털 안보를 설계하고 사이버보안 인재 양성의 방향을 제시한 뜻깊은 자리였다”라며 “세종시가 글로벌 사이버보안 협력의 중심지로 성장할 수 있도록 지원을 아끼지 않겠다”라고 말했다.
+한편, 이번 행사는 시와 국가정보원이 공동 주최하고 고려대 세종(정보보호특성화대학·SW중심대학사업단·RISE사업단)과 홍익대 세종(RISE사업단), 방산기술보호연구소, 한국과학기술정보연구원이 주관했고, 과기정통부와 행안부, 개인정보보호위원회, 한국전자통신연구원, 한국인터넷진흥원 등 18개 기관이 후원했다.
+공공저작물 자유이용 허락 표시
+'핵테온 세종' AI·사이버보안 협력 중심지로 자리매김 저작물은 공공누리 출처표시 조건( 공공누리 4유형 출처표시 + 상업적 이용금지 + 변경금지 )에 따라 이용할 수 있습니다.
+목록 링크복사
+만족도조사
+만족도 조사
+이 페이지에서 제공하는 정보에 대하여 만족하시나요?
+매우만족 만족 보통 불만족 매우불만족
+만족도조사 내용을 입력하세요
+세종 특별자치시
+고정형·이동형 영상정보처리기기운영·관리 방침
+이메일주소무단수집거부
+오시는길
+뷰어프로그램 다운로드
+홈페이지개선의견
+세종특별자치시 한누리대로 2130 (보람동) (우)30151
+대표전화 (044) 120 (유료, 평일 08:30 ~ 18:30, 토·공휴일 09:00~18:00, 근무시간 외 당직실 연결)</t>
+        </is>
+      </c>
+      <c r="G40" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-21T15:18:03.817822+09:00</t>
+        </is>
+      </c>
+      <c r="H40" s="2" t="inlineStr">
+        <is>
+          <t>인공지능, AI, 사이버보안, 개인정보, 플랫폼</t>
+        </is>
+      </c>
+      <c r="I40" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J40" s="2" t="inlineStr">
+        <is>
+          <t>대메뉴 바로가기
+민원·소통·참여
+여행정보
+세종소개
+정보공개
+분야별정보
+생활정보
+로그인
+회원가입
+SNS
+Languages
+세종특별자치시 세종소개
+전체메뉴
+세종소개
+세종소식
+부서바로가기
+세종소식
+시정소식
+고시/공고
+언론보도자료
+해명자료
+영상자료
+세종사진관
+언론보도자료
+HOME
+세종소식
+언론보도자료
+공유 프린트 짧은URL즐겨찾기
+'핵테온 세종' AI·사이버보안 협력 중심지로 자리매김
+작성자인공지능디지털담당관  조회수138
+등록일2026-07-10
+아이콘
+2026_핵테온_세종(인공지능디지털담당관).JPG [1,706.6 KB]
+아이콘
+2026_핵테온_세종2(인공지능디지털담당관).JPG [1,650.5 KB]
+아이콘
+국제_대학생_사이버보안_경진대회(인공지능디지털담당관).JPG [1,958.9 KB]
+한글 아이콘
+추가260710_핵테온세종(인공지능디지털담당관).HWP [242.8 KB] 추가260710_핵테온세종(인공지능디지털담당관).hwp바로보기
+'핵테온 세종' AI·사이버보안 협력 중심지로 자리매김
+- 국가정보원 공동주최로 위상 강화…47개국 5,000여 명 참여 -
+인재 양성·기술 교류·정책 협력 아우른 융합 플랫폼으로 안착 -
+전 세계 사이버보안 인재와 인공지능 보안 기술·정책 역량이 한 데 모인 ‘2026 핵테온 세종’이 이틀간의 대장정을 성공적으로 마쳤다. 세종특별자치시(시장 조상호)는 지난 9∼10일 정부세종컨벤션센터에서 국가정보원과 공동으로 ‘2026 핵테온 세종’을 개최했다. 올해 5회째를 맞은 이번 행사는 국가 차원의 사이버안보 협력 행사로 의미를 더한 가운데 국내외 보안 전문가와 대학생, 기업 관계자 등 5,000여 명이 참여해 인공지능 시대 사이버보안의 해법을 모색했다.</t>
+        </is>
+      </c>
+      <c r="K40" s="2" t="inlineStr">
+        <is>
+          <t>정부부처·청·위원회</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="2" t="inlineStr">
+        <is>
+          <t>15_B000000157517Yy7cB8i</t>
+        </is>
+      </c>
+      <c r="B41" s="2" t="inlineStr">
+        <is>
+          <t>시민 체감형 AI 혁신 아이디어 한자리에</t>
+        </is>
+      </c>
+      <c r="C41" s="2" t="inlineStr">
+        <is>
+          <t>세종특별자치시</t>
+        </is>
+      </c>
+      <c r="D41" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="E41" s="2" t="inlineStr">
+        <is>
+          <t>https://www.sejong.go.kr/bbs/R0079/view.do?nttId=B000000157517Yy7cB8i&amp;mno=sub02_0401&amp;cmsNoStr=&amp;pageIndex=1&amp;kind=</t>
+        </is>
+      </c>
+      <c r="F41" s="2" t="inlineStr">
+        <is>
+          <t>대메뉴 바로가기
+민원·소통·참여
+여행정보
+세종소개
+정보공개
+분야별정보
+생활정보
+로그인
+회원가입
+SNS
+Languages
+세종특별자치시 세종소개
+전체메뉴
+세종소개
+세종소식
+부서바로가기
+세종소식
+시정소식
+고시/공고
+언론보도자료
+해명자료
+영상자료
+세종사진관
+언론보도자료
+HOME
+세종소식
+언론보도자료
+공유 프린트 짧은URL즐겨찾기
+시민 체감형 AI 혁신 아이디어 한자리에
+작성자인공지능디지털담당관  조회수136
+등록일2026-07-10
+아이콘
+AI_혁신_경진대회_수상결과(인공지능디지털담당관).JPG [337.7 KB]
+한글 아이콘
+추가_260710_AI_혁신_경진대회_성료(인공지능디지털담당관).HWP [226.5 KB] 추가_260710_AI_혁신_경진대회_성료(인공지능디지털담당관).hwp바로보기
+시민 체감형 AI 혁신 아이디어 한자리에
+- '제1회 AI 혁신 경진대회' 성료, 도심 공실 해결 아이디어 수상 영예 -
+인공지능(AI)을 활용해 행정 혁신과 도시문제 해결 아이디어를 발굴하기 위해 열린 ‘제1회 세종특별자치시 AI 혁신 경진대회’가 시민들의 뜨거운 관심 속에 마무리됐다.
+세종특별자치시(시장 조상호)는 10일 세종컨벤션센터에서 ‘AI와 함께 도약하는 세종, 시민의 내일을 설계하다’를 표어로, ‘제1회 세종특별자치시 AI 혁신 경진대회’를 개최했다.
+이날 본선에는 예선을 통과한 총 12개 팀이 참가해 전국민 대상 ‘AI 혁신 아이디어 공모전’과 공무원 대상 ‘AI 행정 혁신 우수사례·아이디어 경진대회’ 2개 부문에서 열띤 발표가 펼쳐졌다.
+전문가 심사위원단 평가와 시민 현장평가단 선호도 투표를 합산한 결과, 전 국민 공모 부문에서는 ‘AI 기반 세종시 복지 사각지대 연결·사후관리플랫폼 CARE-ON’을 발표한 한혜인씨가 최우수상에 선정됐다.
+'CARE-ON'은 세종시 읍면동의 복지 취약점수를 산출 및 유형화해 공공서비스 자동 추천, 민간자원 위치 기반 매칭, 30일 사후 관리 알림을 제공하는 복지 연결 지원 시스템이다.
+공무원 부문에서는 ‘AI 재난상황관리 플랫폼 세종 SIREN’을 발표한 안주혁 주무관이 최우수상의 영예를 안았다.
+'세종 SIREN'은 재난상황 입력 시 인공지능이 전파문안과 전파대상을 자동 처리해 상황 전파 시간을 평균 10분에서 10초로 단축한 재난상황관리 플랫폼이다.
+시는 수상작의 혁신 아이디어들을 실제 행정 현장에 적용할 수 있는 방안을 모색하고, 우수 사례를 전 부서에 공유해 인공지능을 기반으로 한 행정 혁신을 속도감 있게 추진해나갈 계획이다.
+조상호 세종시장은 “이번 대회는 인공지능이 행정의 효율을 높이고 시민의 삶을 더 편리하게 만들 수 있다는 가능성을 확인한 자리였다”며 “인공지능 대전환 시대를 맞아 세종시가 시민이 체감하는 인공지능 혁신을 실현할 수 있도록 작은 부분에서부터 실질적인 변화를 만들어가겠다”고 말했다.
+공공저작물 자유이용 허락 표시
+시민 체감형 AI 혁신 아이디어 한자리에 저작물은 공공누리 출처표시 조건( 공공누리 4유형 출처표시 + 상업적 이용금지 + 변경금지 )에 따라 이용할 수 있습니다.
+목록 링크복사
+만족도조사
+만족도 조사
+이 페이지에서 제공하는 정보에 대하여 만족하시나요?
+매우만족 만족 보통 불만족 매우불만족
+만족도조사 내용을 입력하세요
+세종 특별자치시
+고정형·이동형 영상정보처리기기운영·관리 방침
+이메일주소무단수집거부
+오시는길
+뷰어프로그램 다운로드
+홈페이지개선의견
+세종특별자치시 한누리대로 2130 (보람동) (우)30151
+대표전화 (044) 120 (유료, 평일 08:30 ~ 18:30, 토·공휴일 09:00~18:00, 근무시간 외 당직실 연결)</t>
+        </is>
+      </c>
+      <c r="G41" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-21T15:18:13.746139+09:00</t>
+        </is>
+      </c>
+      <c r="H41" s="2" t="inlineStr">
+        <is>
+          <t>AI, 인공지능, 플랫폼</t>
+        </is>
+      </c>
+      <c r="I41" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J41" s="2" t="inlineStr">
+        <is>
+          <t>대메뉴 바로가기
+민원·소통·참여
+여행정보
+세종소개
+정보공개
+분야별정보
+생활정보
+로그인
+회원가입
+SNS
+Languages
+세종특별자치시 세종소개
+전체메뉴
+세종소개
+세종소식
+부서바로가기
+세종소식
+시정소식
+고시/공고
+언론보도자료
+해명자료
+영상자료
+세종사진관
+언론보도자료
+HOME
+세종소식
+언론보도자료
+공유 프린트 짧은URL즐겨찾기
+시민 체감형 AI 혁신 아이디어 한자리에
+작성자인공지능디지털담당관  조회수136
+등록일2026-07-10
+아이콘
+AI_혁신_경진대회_수상결과(인공지능디지털담당관).JPG [337.7 KB]
+한글 아이콘
+추가_260710_AI_혁신_경진대회_성료(인공지능디지털담당관).HWP [226.5 KB] 추가_260710_AI_혁신_경진대회_성료(인공지능디지털담당관).hwp바로보기
+시민 체감형 AI 혁신 아이디어 한자리에
+- '제1회 AI 혁신 경진대회' 성료, 도심 공실 해결 아이디어 수상 영예 -
+인공지능(AI)을 활용해 행정 혁신과 도시문제 해결 아이디어를 발굴하기 위해 열린 ‘제1회 세종특별자치시 AI 혁신 경진대회’가 시민들의 뜨거운 관심 속에 마무리됐다. 세종특별자치시(시장 조상호)는 10일 세종컨벤션센터에서 ‘AI와 함께 도약하는 세종, 시민의 내일을 설계하다’를 표어로, ‘제1회 세종특별자치시 AI 혁신 경진대회’를 개최했다. 이날 본선에는 예선을 통과한 총 12개 팀이 참가해 전국민 대상 ‘AI 혁신 아이디어 공모전’과 공무원 대상 ‘AI 행정 혁신 우수사례·아이디어 경진대회’ 2개 부문에서 열띤 발표가 펼쳐졌다.</t>
+        </is>
+      </c>
+      <c r="K41" s="2" t="inlineStr">
+        <is>
+          <t>정부부처·청·위원회</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="2" t="inlineStr">
+        <is>
+          <t>18_156770344</t>
+        </is>
+      </c>
+      <c r="B42" s="2" t="inlineStr">
+        <is>
+          <t>[보도자료] 국무총리실, AI 아침 강연 개최</t>
+        </is>
+      </c>
+      <c r="C42" s="2" t="inlineStr">
+        <is>
+          <t>국무조정실</t>
+        </is>
+      </c>
+      <c r="D42" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="E42" s="2" t="inlineStr">
+        <is>
+          <t>https://www.korea.kr/briefing/pressReleaseView.do?newsId=156770344&amp;pageIndex=1&amp;repCodeType=&amp;repCode=&amp;startDate=2025-07-13&amp;endDate=2026-07-13&amp;srchWord=AI&amp;period=year</t>
+        </is>
+      </c>
+      <c r="F42" s="2" t="inlineStr">
+        <is>
+          <t>청와대 소식
+공직메일
+알림설정OFF
+상세검색
+[보도자료] 국무총리실, AI 아침 강연 개최
+2026.07.10 국무조정실
+첨부파일
+260710_AI 아침 강연 개최 보도자료.hwpx
+260710_AI 아침 강연 개최 보도자료.pdf
+“이 자료는 국무조정실의 보도자료를 전재하여 제공함을 알려드립니다.”
+법무부, 교정시설 신축에 '공모제' 최초 도입
+포용과 통합의 노사파트너십, 내일의 성장을 이끌다.
+이 대통령 "부동산 조세 제도, 국민의 상식과 눈높이에 기초해 정비"
+식비 줄이는 방법을 모른다고?
+"화장실 갈 시간도 없어요" 국민신문고 민원 처리하는 공정위 직원의 REAL 하루
+AI에게 가장 대체되기 쉬운 사람 양산하는 사회
+국내 첫 세계유산위원회 부산 개막…대한민국 주도 '부산 선언' 채택
+필요한 순간, 필요한 만큼 [ㅅㄱㅈㅂㅇ] 이 필요해요~
+정부, 550조 AI 데이터센터 투자 견인…'1인 1 AI 에이전트' 시대 연다
+하반기 3% 이내 물가관리 총력…3대 메가프로젝트 역량 집중
+잠재성장률 3%·수출 4강·국민소득 5만 달러…'경제 대도약 원년'
+단일종목 레버리지 상품 신규 출시 잠정 중단…예탁금은 현금 3000만 원으로 상향
+국내 첫 세계유산위원회 부산 개막…대한민국 주도 '부산 선언' 채택
+최신뉴스
+식비 줄이는 방법을 모른다고?
+우베만 찾아서 참다 못 해 나왔다! 참, 마!
+기능성표시식품 VS 건강기능식품, 둘의 차이점은?
+호우 대처상황 점검회의
+정책포커스
+기획예산처 (보도설명) 지방교육재정 교부금 개편 관련 구체적인 내용은 결정된 바 없습니다. 2026.07.21
+기획예산처 (보도설명) 지방교육재정 교부금 개편 관련 구체적인 내용은 결정된 바 없습니다. 2026.07.21
+정책브리핑 RSS 서비스 제공 중단 안내
+(30119) 세종특별자치시 갈매로 388 정부세종청사 15동 © 문화체육관광부
+X 바로가기
+네이버포스트 바로가기
+유튜브 바로가기
+인스타그램 바로가기
+행정부처 바로가기</t>
+        </is>
+      </c>
+      <c r="G42" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-21T15:18:21.691534+09:00</t>
+        </is>
+      </c>
+      <c r="H42" s="2" t="inlineStr">
+        <is>
+          <t>AI, 데이터</t>
+        </is>
+      </c>
+      <c r="I42" s="2" t="n">
+        <v>0.628</v>
+      </c>
+      <c r="J42" s="2" t="inlineStr">
+        <is>
+          <t>청와대 소식
+공직메일
+알림설정OFF
+상세검색
+[보도자료] 국무총리실, AI 아침 강연 개최
+2026.07.10 국무조정실
+첨부파일
+260710_AI 아침 강연 개최 보도자료.hwpx
+260710_AI 아침 강연 개최 보도자료.pdf
+“이 자료는 국무조정실의 보도자료를 전재하여 제공함을 알려드립니다.”
+법무부, 교정시설 신축에 '공모제' 최초 도입
+포용과 통합의 노사파트너십, 내일의 성장을 이끌다. 이 대통령 "부동산 조세 제도, 국민의 상식과 눈높이에 기초해 정비"
+식비 줄이는 방법을 모른다고? "화장실 갈 시간도 없어요" 국민신문고 민원 처리하는 공정위 직원의 REAL 하루
+AI에게 가장 대체되기 쉬운 사람 양산하는 사회
+국내 첫 세계유산위원회 부산 개막…대한민국 주도 '부산 선언' 채택
+필요한 순간, 필요한 만큼 [ㅅㄱㅈㅂㅇ] 이 필요해요~
+정부, 550조 AI 데이터센터 투자 견인…'1인 1 AI 에이전트' 시대 연다
+하반기 3% 이내 물가관리 총력…3대 메가프로젝트 역량 집중
+잠재성장률 3%·수출 4강·국민소득 5만 달러…'경제 대도약 원년'
+단일종목 레버리지 상품 신규 출시 잠정 중단…예탁금은 현금 3000만 원으로 상향
+국내 첫 세계유산위원회 부산 개막…대한민국 주도 '부산 선언' 채택
+최신뉴스
+식비 줄이는 방법을 모른다고?</t>
+        </is>
+      </c>
+      <c r="K42" s="2" t="inlineStr">
+        <is>
+          <t>정부부처·청·위원회</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="2" t="inlineStr">
+        <is>
+          <t>1_461355</t>
+        </is>
+      </c>
+      <c r="B43" s="2" t="inlineStr">
+        <is>
+          <t>(석간) DDP, AI 웰니스 로봇 만나 스마트 디자인 공간으로 진화된다</t>
+        </is>
+      </c>
+      <c r="C43" s="2" t="inlineStr">
+        <is>
+          <t>서울특별시</t>
+        </is>
+      </c>
+      <c r="D43" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="E43" s="2" t="inlineStr">
+        <is>
+          <t>https://www.seoul.go.kr/news/news_report.do#view/461355</t>
+        </is>
+      </c>
+      <c r="F43" s="2" t="inlineStr">
+        <is>
+          <t>HOME
+서울소식
+보도·해명자료
+본문 글자 크기 크게 변경
+본문 글자 크기 작게 변경
+(석간) DDP, AI 웰니스 로봇 만나 스마트 디자인 공간으로 진화된다
+서울디자인재단 서울디자인재단
+등록일
+2026-07-10
+수정일
+2026-07-10
+첨부파일
+바로듣기
+첨부파일
+(석간) DDP, AI 웰니스 로봇 만나 스마트 디자인 공간으로 진화된다.hwp
+(75 MB Bytes, 다운로드: 216 회 )
+DDP, AI 웰니스 로봇 만나 스마트 디자인 공간으로 진화된다
+- 서울디자인재단 · SK인텔릭스 ‘DDP 스마트 디자인 환경 조성’ 업무협약 체결
+- DDP 곳곳 ‘나무엑스’ 로봇으로 공기관리, 건강상태 등 생활밀착형 스마트 서비스 경험
+- 양사 디자인 사업과 콘텐츠 연계, 서울의 디자인 경쟁력과 AI기술의 확산 유도
+- 공공 디자인 플랫폼 DDP가 AI 로봇 기술의 실증 무대가 되도록 지원할 것
+전시를 보러 온 방문객이
+로봇에게 길을 묻고
+로봇 앞에서 자신의 건강 상태를 간편하게 확인한다
+공간을 이동하는 로봇은 실내 공기를 관리하며 쾌적한 관람 환경을 만든다
+서울의 대표 디자인 플랫폼
+DDP(
+동대문디자인플라자
+가 디자인과 첨단기술이 결합한 스마트 디자인 플랫폼으로 진화하고 있다
+서울디자인재단
+대표이사 차강희
+이하 재단
+은 지난
+인텔릭스
+대표이사 안무인
+서울시 디자인 산업 발전 및
+DDP
+스마트 디자인 환경 조성을 위한 업무협약
+을 체결하고
+DDP
+를 시민이 미래기술을 가장 먼저 경험하는 공공 디자인 테스트 베드
+(Test Bed)
+로 조성하기 위한 협력에 나섰다
+이번 협약은
+DDP
+에서 전시나 행사 공간을 찾을 시 움직이는
+로봇을 통해 방향을 찾고 깨끗한 공기를 마시게 되는 등 디자인 공간에서 시민의 경험을 혁신하는 것이다
+○ 이를 위해 재단은 SK인텔릭스의 AI 웰니스 로봇 ‘나무엑스(NAMUHX)’를 DDP에 도입한다. 나무엑스는 자율주행 기반 에어 솔루션과 비접촉 컨디션 체크 기능 등을 갖춘 웰니스 로봇으로, DDP 방문객에게 공기 관리, 건강 상태 확인 등 생활밀착형 스마트 서비스를 제공할 예정이다.
+방문객들은
+DDP
+곳곳을 이동하는
+웰니스 로봇
+나무엑스
+를 통해 공기질 관리 서비스를 제공받고
+비접촉 방식으로 자신의 컨디션을 간편하게 확인하는 등 새로운 방식의 웰니스 서비스를 경험할 수 있다
+○ 이는 공간을 아름답게 만드는 디자인에서 시민의 경험과 건강, 편의를 함께 고려하는 미래형 디자인 모델이라는 점에서 의미가 있다.
+양 기관은 이번 협약을 계기로
+DDP
+를 거점으로 한 디자인 산업의 미래 가치 창출
+웰니스 로봇 나무엑스를 활용한 스마트 디자인 환경 조성
+양 기관 디자인 사업 및 콘텐츠의 유기적 연계
+오프라인 공동 홍보 및 마케팅
+기타 디자인 산업 활성화를 위한 협력 과제 등을 함께 추진한다
+안무인
+인텔릭스 대표이사는
+세계 최초의 웰니스 로봇 나무엑스가 서울의 상징적인 디자인 랜드마크인
+DDP
+와 만나 새로운 시너지를 낼 것으로 기대한다
+, “
+에이전틱
+AI(Agentic AI)
+기술을 바탕으로 고객의 일상을 더욱 풍요롭게 만드는 회사가 될 수 있도록 노력하겠다
+고 밝혔다
+차강희 서울디자인재단 대표이사는
+“DDP
+는 서울의 디자인 콘텐츠를 시민과 세계에 연결하는 공공 디자인 플랫폼이자
+미래 산업의 가능성을 실험하는 공간
+이라며
+이번 협약을 계기로 디자인과
+가 융합된 스마트 디자인 경험을 확대하고 서울 디자인 산업의 미래 가치를 확산해 나가겠다
+고 화답했다
+한편 재단은
+기반 공간 서비스에 이어 콘텐츠 분야로 미래 기술을 확대한다
+올해 하반기에는
+넥스트 크리에이티브 페스티벌
+이 열릴 예정이다
+이 행사는
+DDP
+중심의 야간 활성화 거점을 구축하고
+융복합 디자인 산업을 육성하기 위해 기획된 페스티벌이다
+○ 주요 프로그램으로는 시민 참여형 서울 디자인 AI 영상 공모전, 야간 미디어파사드 상영, 기술 융합 포럼 등이 마련됐다. 서울디자인재단은 AI·AR·버추얼 등 최신 엔터테크(기술 융합)를 접목한 이번 축제를 통해 콘텐츠 산업과 관광, 동대문 상권을 동시에 활성화하고 ‘AI 선도 도시, 서울’의 브랜드 가치를 높일 계획이다.
+서울디자인재단
+·SK
+인텔릭스 협약 사진
+서울디자인재단
+·SK
+인텔릭스 협약식 개요 및 주요 내용
+본 저작물은 "공공누리"
+제4유형:출처표시+상업적 이용금지+변경금지
+조건에 따라 이용 할 수 있습니다.
+글퍼가기
+페이지 만족도 조사
+이 페이지에서 제공하는 정보에 대하여 만족하십니까?
+아니오
+5점 - 매우만족
+4점 - 만족
+3점 - 보통
+2점 - 불만족
+1점 - 매우 불만족
+평가하기</t>
+        </is>
+      </c>
+      <c r="G43" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-21T15:18:31.648897+09:00</t>
+        </is>
+      </c>
+      <c r="H43" s="2" t="inlineStr">
+        <is>
+          <t>로봇, AI, 자율주행, 플랫폼</t>
+        </is>
+      </c>
+      <c r="I43" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J43" s="2" t="inlineStr">
+        <is>
+          <t>HOME
+서울소식
+보도·해명자료
+본문 글자 크기 크게 변경
+본문 글자 크기 작게 변경
+(석간) DDP, AI 웰니스 로봇 만나 스마트 디자인 공간으로 진화된다
+서울디자인재단 서울디자인재단
+등록일
+2026-07-10
+수정일
+2026-07-10
+첨부파일
+바로듣기
+첨부파일
+(석간) DDP, AI 웰니스 로봇 만나 스마트 디자인 공간으로 진화된다.hwp
+(75 MB Bytes, 다운로드: 216 회 )
+DDP, AI 웰니스 로봇 만나 스마트 디자인 공간으로 진화된다
+- 서울디자인재단 · SK인텔릭스 ‘DDP 스마트 디자인 환경 조성’ 업무협약 체결
+- DDP 곳곳 ‘나무엑스’ 로봇으로 공기관리, 건강상태 등 생활밀착형 스마트 서비스 경험
+- 양사 디자인 사업과 콘텐츠 연계, 서울의 디자인 경쟁력과 AI기술의 확산 유도
+- 공공 디자인 플랫폼 DDP가 AI 로봇 기술의 실증 무대가 되도록 지원할 것
+전시를 보러 온 방문객이
+로봇에게 길을 묻고
+로봇 앞에서 자신의 건강 상태를 간편하게 확인한다
+공간을 이동하는 로봇은 실내 공기를 관리하며 쾌적한 관람 환경을 만든다
+서울의 대표 디자인 플랫폼
+DDP(
+동대문디자인플라자
+가 디자인과 첨단기술이 결합한 스마트 디자인 플랫폼으로 진화하고 있다
+서울디자인재단
+대표이사 차강희
+이하 재단
+은 지난
+인텔릭스
+대표이사 안무인
+서울시 디자인 산업 발전 및
+DDP
+스마트 디자인 환경 조성을 위한 업무협약
+을 체결하고
+DDP
+를 시민이 미래기술을 가장 먼저 경험하는 공공 디자인 테스트 베드
+(Test Bed)
+로 조성하기 위한 협력에 나섰다
+이번 협약은
+DDP
+에서 전시나 행사 공간을 찾을 시 움직이는
+로봇을 통해 방향을 찾고 깨끗한 공기를 마시게 되는 등 디자인 공간에서 시민의 경험을 혁신하는 것이다
+○ 이를 위해 재단은 SK인텔릭스의 AI 웰니스 로봇 ‘나무엑스(NAMUHX)’를 DDP에 도입한다. 나무엑스는 자율주행 기반 에어 솔루션과 비접촉 컨디션 체크 기능 등을 갖춘 웰니스 로봇으로, DDP 방문객에게 공기 관리, 건강 상태 확인 등 생활밀착형 스마트 서비스를 제공할 예정이다. 방문객들은
+DDP
+곳곳을 이동하는
+웰니스 로봇
+나무엑스
+를 통해 공기질 관리 서비스를 제공받고
+비접촉 방식으로 자신의 컨디션을 간편하게 확인하는 등 새로운 방식의 웰니스 서비스를 경험할 수 있다
+○ 이는 공간을 아름답게 만드는 디자인에서 시민의 경험과 건강, 편의를 함께 고려하는 미래형 디자인 모델이라는 점에서 의미가 있다.</t>
+        </is>
+      </c>
+      <c r="K43" s="2" t="inlineStr">
+        <is>
+          <t>정부부처·청·위원회</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="2" t="inlineStr">
+        <is>
+          <t>1_461401</t>
+        </is>
+      </c>
+      <c r="B44" s="2" t="inlineStr">
+        <is>
+          <t>“AI가 대체 못 하는 역량, 자원봉사에서 배운다”…서울시자원봉사센터, 기업 연계 진로 멘토링 운영</t>
+        </is>
+      </c>
+      <c r="C44" s="2" t="inlineStr">
+        <is>
+          <t>서울특별시</t>
+        </is>
+      </c>
+      <c r="D44" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="E44" s="2" t="inlineStr">
+        <is>
+          <t>https://www.seoul.go.kr/news/news_report.do#view/461401</t>
+        </is>
+      </c>
+      <c r="F44" s="2" t="inlineStr">
+        <is>
+          <t>HOME
+서울소식
+보도·해명자료
+본문 글자 크기 크게 변경
+본문 글자 크기 작게 변경
+“AI가 대체 못 하는 역량, 자원봉사에서 배운다”…서울시자원봉사센터, 기업 연계 진로 멘토링 운영
+서울시자원봉사센터 서울시자원봉사센터
+등록일
+2026-07-10
+수정일
+2026-07-10
+첨부파일
+바로듣기
+첨부파일
+“AI가 대체 못 하는 역량, 자원봉사에서 배운다”… 서울시자원봉사센터, 기업 연계 진로 멘토링 운영.hwp
+(11 MB Bytes, 다운로드: 199 회 )
+“AI가 대체 못 하는 역량, 자원봉사에서 배운다”…서울시자원봉사센터, 기업 연계 진로 멘토링 운영
+- 서울 청년 대상 현직자 재능기부 진로 멘토링 ‘청춘잡담(Job Talk)’ 운영
+- 진로 탐색부터 기업 현장 체험까지 단계별 커리어 멘토링 지원
+- KAIST 서용석 교수 ‘AI 시대, 미래 역량과 커리어 전략’ 특별강연 진행
+서울시자원봉사센터
+센터장 송창훈
+는 지난
+숙명여자대학교에서
+서울 소재 기업
+기관 현직자
+170
+명이 참여한 진로 멘토링 프로그램
+청춘잡담
+(Job Talk)’
+을 진행했다
+○ AI 기술 확산과 사회 변화 속에서 청년들의 진로 불안과 미래 역량에 대한 고민이 커지는 가운데, 서울시자원봉사센터는 청년과 현직자가 직접 만나 경험과 고민을 나누는 관계형 진로 멘토링 프로그램을 운영하고 있다.
+○ ‘청춘잡담’은 다양한 분야의 현직 멘토와 청년 멘티가 직접 만나 직무와 진로에 대한 경험을 나누는 멘토링 프로그램으로, 만 19세~34세 청년이라면 누구나 참여할 수 있다.
+청춘잡담
+(Job Talk)’
+은 진로 탐색을 위한
+차 멘토링과 기업
+기관 업무 현장 체험이 가능한
+차 멘토링으로 나누어 운영된다
+○ 1차 멘토링에서는 특별강연과 멘토-멘티 대화를 통해 진로 방향과 관심 분야를 탐색하고, 2차 멘토링에서는 기업·기관 현장을 직접 방문해 실제 업무 환경과 조직문화를 경험하는 시간을 갖는다.
+○ 멘토들은 단순한 정보 전달자가 아니라 청년들의 고민과 방향성을 함께 나누는 대화 파트너이자 현장 가이드로 참여한다.
+이번 진로 멘토링에는
+삼표산업
+서울디자인재단
+서울문화재단
+에쓰오일
+한국문화예술교육진흥원 등 서울 소재
+개 기업
+공공기관
+재단 소속 임직원
+명이 멘토로 참여하여 직무 경험과 커리어 과정
+조직문화
+사회생활 경험 등을 공유하였다
+○ 이번 프로그램은 단순한 취업 정보 전달 중심이 아니라 청년과 현직자가 서로의 고민과 경험을 나누는 소통 중심 프로그램으로 운영된다.
+○ 참여 청년들은 서울 청년 기획봉사단 및 대학연계 프로젝트 참여자를 포함해 기후위기, 교육 격차, 공동체 회복 등 다양한 사회문제에 관심을 가지고 활동 중인 청년들로, 이번 멘토링을 통해 자신의 관심사와 사회참여 경험을 진로와 연결해보는 시간을 가졌다.
+숙명여자대학교에서 진행된
+차 멘토링은 청년을 위한 특별강연을 시작으로
+같은 고민을 가진 청년 간 네트워크 형성
+멘티 간 만남
+질의응답 등 약
+시간에 걸쳐 진행되었다
+○ 매칭된 멘토와 멘티는 상호 자기소개를 시작으로 직무와 진로에 대한 고민을 공유하고, 현직자의 생생한 경험과 정보를 나누는 시간을 가졌다.
+특히 이번 특별강연에는
+KAIST
+문술미래전략대학원 교수이자 미래전략연구센터장인 서용석 교수가 참여해
+대전환 시대의 사회 변화와 청년에게 필요한 미래 역량을 주제로 강연을 진행했다
+○ 서용석 교수는 ‘AI시대, 미래학자가 연구한 미래 직업과 필수 역량’을 주제로 ▲AI 기술이 가져올 산업과 직무의 변화, ▲AI 시대의 새로운 커리어 전략, ▲기술 문해력과 적응력, ▲창의성과 공감 등 미래 사회에서 요구되는 핵심 역량에 대해 강연하였다. 또한 AI는 인간의 일을 단순히 대체하는 것이 아니라 업무를 재구성하는 만큼, 청년들이 직무 자체보다 문제 해결 역량과 자신만의 경험을 바탕으로 경쟁력을 갖추는 것이 중요하다고 강조했다.
+○ 이어 급변하는 기술 환경 속에서 청년들이 변화에 유연하게 적응하고, 인간만이 발휘할 수 있는 창의성과 공감, 가치 판단 능력을 바탕으로 자신만의 경쟁력을 키워나가야 한다는 메시지를 전했다.
+송창훈 서울시자원봉사센터장은
+청춘잡담은 단순한 취업 지원 프로그램이 아니라
+청년들이 다양한 현직자와 만나 자신의 경험과 고민을 연결해보는 과정
+이라며
+, “
+앞으로도 청년들의 사회참여 경험이 성장과 진로로 이어질 수 있도록 다양한 연계 프로그램을 운영해 나가겠다
+고 밝혔다
+, ‘
+청춘잡담
+(Job Talk)’
+은 지난
+) 1
+차 멘토링을 성황리에 마쳤으며
+까지 기업
+기관별
+차 멘토링을 순차적으로 진행한다
+자세한 내용은 서울동행 누리집에서 확인할 수 있다
+본 저작물은 "공공누리"
+제4유형:출처표시+상업적 이용금지+변경금지
+조건에 따라 이용 할 수 있습니다.
+글퍼가기
+페이지 만족도 조사
+이 페이지에서 제공하는 정보에 대하여 만족하십니까?
+아니오
+5점 - 매우만족
+4점 - 만족
+3점 - 보통
+2점 - 불만족
+1점 - 매우 불만족
+평가하기</t>
+        </is>
+      </c>
+      <c r="G44" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-21T15:18:41.637722+09:00</t>
+        </is>
+      </c>
+      <c r="H44" s="2" t="inlineStr">
+        <is>
+          <t>AI</t>
+        </is>
+      </c>
+      <c r="I44" s="2" t="n">
+        <v>0.386</v>
+      </c>
+      <c r="J44" s="2" t="inlineStr">
+        <is>
+          <t>HOME
+서울소식
+보도·해명자료
+본문 글자 크기 크게 변경
+본문 글자 크기 작게 변경
+“AI가 대체 못 하는 역량, 자원봉사에서 배운다”…서울시자원봉사센터, 기업 연계 진로 멘토링 운영
+서울시자원봉사센터 서울시자원봉사센터
+등록일
+2026-07-10
+수정일
+2026-07-10
+첨부파일
+바로듣기
+첨부파일
+“AI가 대체 못 하는 역량, 자원봉사에서 배운다”… 서울시자원봉사센터, 기업 연계 진로 멘토링 운영.hwp
+(11 MB Bytes, 다운로드: 199 회 )
+“AI가 대체 못 하는 역량, 자원봉사에서 배운다”…서울시자원봉사센터, 기업 연계 진로 멘토링 운영
+- 서울 청년 대상 현직자 재능기부 진로 멘토링 ‘청춘잡담(Job Talk)’ 운영
+- 진로 탐색부터 기업 현장 체험까지 단계별 커리어 멘토링 지원
+- KAIST 서용석 교수 ‘AI 시대, 미래 역량과 커리어 전략’ 특별강연 진행
+서울시자원봉사센터
+센터장 송창훈
+는 지난
+숙명여자대학교에서
+서울 소재 기업
+기관 현직자
+170
+명이 참여한 진로 멘토링 프로그램
+청춘잡담
+(Job Talk)’
+을 진행했다
+○ AI 기술 확산과 사회 변화 속에서 청년들의 진로 불안과 미래 역량에 대한 고민이 커지는 가운데, 서울시자원봉사센터는 청년과 현직자가 직접 만나 경험과 고민을 나누는 관계형 진로 멘토링 프로그램을 운영하고 있다. ○ ‘청춘잡담’은 다양한 분야의 현직 멘토와 청년 멘티가 직접 만나 직무와 진로에 대한 경험을 나누는 멘토링 프로그램으로, 만 19세~34세 청년이라면 누구나 참여할 수 있다. 청춘잡담
+(Job Talk)’
+은 진로 탐색을 위한
+차 멘토링과 기업
+기관 업무 현장 체험이 가능한
+차 멘토링으로 나누어 운영된다
+○ 1차 멘토링에서는 특별강연과 멘토-멘티 대화를 통해 진로 방향과 관심 분야를 탐색하고, 2차 멘토링에서는 기업·기관 현장을 직접 방문해 실제 업무 환경과 조직문화를 경험하는 시간을 갖는다.</t>
+        </is>
+      </c>
+      <c r="K44" s="2" t="inlineStr">
+        <is>
+          <t>정부부처·청·위원회</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="2" t="inlineStr">
+        <is>
+          <t>13_42397259</t>
+        </is>
+      </c>
+      <c r="B45" s="2" t="inlineStr">
+        <is>
+          <t>경남도, 전국 최초 ‘피지컬AI 고속도로’ 구축 본격화</t>
+        </is>
+      </c>
+      <c r="C45" s="2" t="inlineStr">
+        <is>
+          <t>경상남도</t>
+        </is>
+      </c>
+      <c r="D45" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="E45" s="2" t="inlineStr">
+        <is>
+          <t>https://www.gyeongnam.go.kr/board/view.gyeong?boardId=BBS_0000060&amp;menuCd=DOM_000000135002001000&amp;paging=ok&amp;startPage=1&amp;searchType=DATA_TITLE&amp;searchOperation=AND&amp;keyword=AI&amp;categoryCode1=A&amp;dataSid=42397259</t>
+        </is>
+      </c>
+      <c r="F45" s="2" t="inlineStr">
+        <is>
+          <t>경남소식
+보도해명자료
+경남도, 전국 최초 ‘피지컬AI 고속도로’ 구축 본격화
+조회 :
+391
+등록일 :
+26.07.10
+제공부서
+인공지능산업과
+담당자
+손창환 사무관, 이상훈 주무관
+전화번호
+055-211-3972, 055-211-3973
+부제목
+- 전국 최초 산단전용 5G 특화망 구축사업 선정…국비 105억 원 확보 - AX실증산단에 이어 피지컬AI 핵심 인프라 데이터 고속도로 구축 - 민선 9기 도정 핵심전략 ‘글로벌 피지컬AI 수도 경남’ 실현 가속화
+첨부파일
+0710보도자료(산단전용 5G특화망 구축-창원국가산단 공모 선정)-인공지능산업과.hwp (1084 kb)
+바로듣기
+0710보도자료(산단전용 5G특화망 구축-창원국가산단 공모 선정)-인공지능산업과.hwpx (1081 kb)
+바로듣기
+경남도청 전경.jpg (10170 kb)
+경남도
+전국 최초
+피지컬
+고속도로
+구축 본격화
+전국 최초 산단전용
+특화망 구축사업 선정
+105
+억 원 확보
+- AX
+실증산단에 이어 피지컬
+핵심 인프라 데이터 고속도로 구축
+기 도정 핵심전략
+글로벌 피지컬
+수도 경남
+실현 가속화
+경상남도
+도지사 박완수
+는 산업통상부가 추진하는
+산단전용
+특화망 구축사업
+공모에서 창원국가산업단지가 전국
+개 스마트그린산단 가운데 유일하게 최종 선정돼 국비
+105
+억 원을 확보했다고 밝혔다
+이번 사업은 지난해 선정돼 추진 중인 창원국가산단
+실증산단 구축사업과 오는
+월 개소 예정인 피지컬
+원스톱 지원 플랫폼
+경남제조
+데이터센터 등을 하나로 연결하는 피지컬
+핵심 인프라 구축사업이다
+이를 통해 피지컬
+가 도내 제조현장에서 실시간으로 작동할 수 있는
+피지컬
+고속도로
+(Physical AI Highway)’
+를 구축하는 전국 최초 시범사업이다
+도는 지난해부터
+글로벌 피지컬
+수도 경남
+실현을 위해 제조현장의 피지컬
+확산에 필수적인
+특화망 구축 필요성을 인식하고
+한국산업단지공단 경남지역본부와 함께 지역 국회의원들과 협력해 정부에 지속적으로 건의해왔다
+그 결과 올해 정부 공모사업으로 반영돼 전국 최초로 시범사업을 유치하는 성과를 거뒀으며
+경남이 정부의 피지컬
+정책을 선도하며 국가
+사업으로 실현시킨 성과라는 점에서 의미가 크다
+피지컬
+수도 경남에서 전국 최초 피지컬
+고속도로 구축 추진
+피지컬
+가 로봇과 제조설비를 통해 산업현장에서 스스로 판단하고 움직이는 차세대 제조혁신 기술로
+피지컬
+가 제대로 작동하기 위해서는
+와 로봇
+제조설비
+데이터센터를 초고속으로 연결하는 통신망 구축이 필수적이다
+이번 사업은 초고속 데이터 고속도로를 구축하는 사업으로 총사업비
+150
+억 원을 투입해 창원국가산단 전역에 기업들이 공동 활용할 수 있는
+특화망을 구축하고
+향후 진주
+사천 등 도내 전역으로 확산할 계획이다
+주요 사업으로 산단 공동 활용형
+5G Core
+와 통합관제센터 구축을 통한
+클라우드 서비스와 공공
+기업특화형 등
+특화망을 활용한
+실증을 지원하며
+이를 통해 제조기업들이 대규모 투자 없이도 대용량의 데이터를 처리할 수 있는 초고속
+서비스 활용으로 현장의 피지컬
+확산을 가속화시킬 수 있다
+실증산단
+경남제조
+데이터센터 등 연계
+경남형 피지컬
+인프라
+경남도는 지난해 선정된 창원국가산단
+실증산단 구축사업과 오는
+월 개소 예정인 피지컬
+원스톱 지원 플랫폼
+경남제조
+데이터센터 등을 유기적으로 연결하는 경남형 피지컬
+지원 인프라를 구축할 계획이다
+피지컬
+는 사람의 몸과 같은 구조로
+로봇은 신체
+(Body),
+피지컬
+파운데이션 모델은 두뇌
+(Brain),
+데이터센터는 심장
+(Heart),
+산업데이터는 혈액
+(Blood), 5G
+특화망은 정보를 실시간으로 전달하는 혈관이자 초고속 신경망
+(Network)
+역할을 한다
+데이터센터에서 학습한
+특화망을 통해 제조현장의 로봇과 설비로 전달되고
+현장에서 생성되는 대용량 데이터는 다시 데이터센터로 전송돼
+가 지속적으로 학습
+고도화되는 선순환 구조를 완성하게 된다
+이번 사업은
+AI·
+데이터
+로봇을 하나로 연결하는 핵심 기반을 구축함으로써 도내제조기업이 피지컬
+를 활용할 수 있는 환경을 마련하는 것은 물론
+경남이 추진하는 제조
+전 주기 생태계를 완성하는 핵심 인프라가 될 것으로 기대한다
+경남형 제조 특화 피지컬
+혁신 벨트
+구축으로 도내 전방위적
+도는 이번 사업을 기반으로 창원국가산단과 사천우주항공국가산단까지 연결하는
+경남형 제조 특화 피지컬
+혁신벨트
+구축으로 기계
+자동차
+조선 등 동
+중부경남의 주력 제조산업과 첨단우주항공산업 중심의 서부경남 제조산업을 하나의 피지컬
+생태계로 연결하고
+검증된 제조
+모델을 경남 전역으로 확산해 민선
+기 도정 핵심 전략인
+글로벌 피지컬
+수도 경남
+실현을 본격화한다는 방침이다
+경남도는 이번 사업으로 피지컬
+와 로봇
+데이터센터를 하나로 연결하는
+전국 최초의 피지컬
+고속도로
+를 본격 구축해 도내 피지컬
+의 전방위적 확산을 추진해 나갈 계획이다
+이미화 경남도 산업국장은
+이번 산단전용
+특화망 구축 사업은 전국 최초 피지컬
+고속도로이자 제조
+혁신을 위한 핵심 인프라로
+경남이 대한민국 제조혁신을 넘어 글로벌 피지컬
+중심지로 도약하는 중요한 전환점이 될 것이다
+, “
+창원국가산단과 사천우주항공국가산단까지 도내 거점 산단을 연결하는 경남형 피지컬
+혁신벨트 구축 확산으로 글로벌 피지컬
+혁신을 선도해 나가겠다
+고 말했다
+이 보도자료와 관련하여 보다 자세한 내용이나 취재를 원하시면 인공지능산업과 손창환 사무관
+(055-211-3972)
+이상훈 주무관
+(055-211-3973)
+에게 연락주시기 바랍니다
+경남도, 전국 최초 ‘피지컬AI 고속도로’ 구축 본격화 저작물은 공공누리 “출처표시+상업적이용금지” 조건에 따라 이용할 수 있습니다.
+경남도, 국토지리정보원과 함께 개발제한구역 아날로그 항공사진 DB 구축 본격 추진
+경남자치경찰위, 여름 휴가철 맞아 ‘찾아가는 안심 지문등록’ 실시
+경상남도 민원 콜센터
+연락처 :
+055-120
+이 페이지에서 제공하는 정보에 대하여 만족하십니까?
+매우만족
+불만족
+매우불만족
+의견 입력하기
+의견 등록하기
+0 / 100</t>
+        </is>
+      </c>
+      <c r="G45" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-21T15:18:48.351261+09:00</t>
+        </is>
+      </c>
+      <c r="H45" s="2" t="inlineStr">
+        <is>
+          <t>AI, 로봇, 인공지능, AX, 파운데이션, 데이터, 플랫폼, 클라우드</t>
+        </is>
+      </c>
+      <c r="I45" s="2" t="n">
+        <v>0.881</v>
+      </c>
+      <c r="J45" s="2" t="inlineStr">
+        <is>
+          <t>경남소식
+보도해명자료
+경남도, 전국 최초 ‘피지컬AI 고속도로’ 구축 본격화
+조회 :
+391
+등록일 :
+26.07.10
+제공부서
+인공지능산업과
+담당자
+손창환 사무관, 이상훈 주무관
+전화번호
+055-211-3972, 055-211-3973
+부제목
+- 전국 최초 산단전용 5G 특화망 구축사업 선정…국비 105억 원 확보 - AX실증산단에 이어 피지컬AI 핵심 인프라 데이터 고속도로 구축 - 민선 9기 도정 핵심전략 ‘글로벌 피지컬AI 수도 경남’ 실현 가속화
+첨부파일
+0710보도자료(산단전용 5G특화망 구축-창원국가산단 공모 선정)-인공지능산업과.hwp (1084 kb)
+바로듣기
+0710보도자료(산단전용 5G특화망 구축-창원국가산단 공모 선정)-인공지능산업과.hwpx (1081 kb)
+바로듣기
+경남도청 전경.jpg (10170 kb)
+경남도
+전국 최초
+피지컬
+고속도로
+구축 본격화
+전국 최초 산단전용
+특화망 구축사업 선정
+105
+억 원 확보
+- AX
+실증산단에 이어 피지컬
+핵심 인프라 데이터 고속도로 구축
+기 도정 핵심전략
+글로벌 피지컬
+수도 경남
+실현 가속화
+경상남도
+도지사 박완수
+는 산업통상부가 추진하는
+산단전용
+특화망 구축사업
+공모에서 창원국가산업단지가 전국
+개 스마트그린산단 가운데 유일하게 최종 선정돼 국비
+105
+억 원을 확보했다고 밝혔다
+이번 사업은 지난해 선정돼 추진 중인 창원국가산단
+실증산단 구축사업과 오는
+월 개소 예정인 피지컬
+원스톱 지원 플랫폼
+경남제조
+데이터센터 등을 하나로 연결하는 피지컬
+핵심 인프라 구축사업이다
+이를 통해 피지컬
+가 도내 제조현장에서 실시간으로 작동할 수 있는
+피지컬
+고속도로
+(Physical AI Highway)’
+를 구축하는 전국 최초 시범사업이다
+도는 지난해부터
+글로벌 피지컬
+수도 경남
+실현을 위해 제조현장의 피지컬
+확산에 필수적인
+특화망 구축 필요성을 인식하고
+한국산업단지공단 경남지역본부와 함께 지역 국회의원들과 협력해 정부에 지속적으로 건의해왔다
+그 결과 올해 정부 공모사업으로 반영돼 전국 최초로 시범사업을 유치하는 성과를 거뒀으며
+경남이 정부의 피지컬
+정책을 선도하며 국가
+사업으로 실현시킨 성과라는 점에서 의미가 크다
+피지컬
+수도 경남에서 전국 최초 피지컬
+고속도로 구축 추진
+피지컬
+가 로봇과 제조설비를 통해 산업현장에서 스스로 판단하고 움직이는 차세대 제조혁신 기술로
+피지컬
+가 제대로 작동하기 위해서는
+와 로봇
+제조설비
+데이터센터를 초고속으로 연결하는 통신망 구축이 필수적이다
+이번 사업은 초고속 데이터 고속도로를 구축하는 사업으로 총사업비
+150
+억 원을 투입해 창원국가산단 전역에 기업들이 공동 활용할 수 있는
+특화망을 구축하고
+향후 진주
+사천 등 도내 전역으로 확산할 계획이다
+주요 사업으로 산단 공동 활용형
+5G Core
+와 통합관제센터 구축을 통한
+클라우드 서비스와 공공
+기업특화형 등
+특화망을 활용한
+실증을 지원하며
+이를 통해 제조기업들이 대규모 투자 없이도 대용량의 데이터를 처리할 수 있는 초고속
+서비스 활용으로 현장의 피지컬
+확산을 가속화시킬 수 있다
+실증산단
+경남제조
+데이터센터 등 연계
+경남형 피지컬
+인프라
+경남도는 지난해 선정된 창원국가산단
+실증산단 구축사업과 오는
+월 개소 예정인 피지컬
+원스톱 지원 플랫폼
+경남제조
+데이터센터 등을 유기적으로 연결하는 경남형 피지컬
+지원 인프라를 구축할 계획이다
+피지컬
+는 사람의 몸과 같은 구조로
+로봇은 신체
+(Body),
+피지컬
+파운데이션 모델은 두뇌
+(Brain),
+데이터센터는 심장
+(Heart),
+산업데이터는 혈액
+(Blood), 5G
+특화망은 정보를 실시간으로 전달하는 혈관이자 초고속 신경망
+(Network)
+역할을 한다
+데이터센터에서 학습한
+특화망을 통해 제조현장의 로봇과 설비로 전달되고
+현장에서 생성되는 대용량 데이터는 다시 데이터센터로 전송돼
+가 지속적으로 학습
+고도화되는 선순환 구조를 완성하게 된다
+이번 사업은
+AI·
+데이터
+로봇을 하나로 연결하는 핵심 기반을 구축함으로써 도내제조기업이 피지컬
+를 활용할 수 있는 환경을 마련하는 것은 물론
+경남이 추진하는 제조
+전 주기 생태계를 완성하는 핵심 인프라가 될 것으로 기대한다
+경남형 제조 특화 피지컬
+혁신 벨트
+구축으로 도내 전방위적
+도는 이번 사업을 기반으로 창원국가산단과 사천우주항공국가산단까지 연결하는
+경남형 제조 특화 피지컬
+혁신벨트
+구축으로 기계
+자동차
+조선 등 동
+중부경남의 주력 제조산업과 첨단우주항공산업 중심의 서부경남 제조산업을 하나의 피지컬
+생태계로 연결하고
+검증된 제조
+모델을 경남 전역으로 확산해 민선
+기 도정 핵심 전략인
+글로벌 피지컬
+수도 경남
+실현을 본격화한다는 방침이다
+경남도는 이번 사업으로 피지컬
+와 로봇
+데이터센터를 하나로 연결하는
+전국 최초의 피지컬
+고속도로
+를 본격 구축해 도내 피지컬
+의 전방위적 확산을 추진해 나갈 계획이다
+이미화 경남도 산업국장은
+이번 산단전용
+특화망 구축 사업은 전국 최초 피지컬
+고속도로이자 제조
+혁신을 위한 핵심 인프라로
+경남이 대한민국 제조혁신을 넘어 글로벌 피지컬
+중심지로 도약하는 중요한 전환점이 될 것이다
+, “
+창원국가산단과 사천우주항공국가산단까지 도내 거점 산단을 연결하는 경남형 피지컬
+혁신벨트 구축 확산으로 글로벌 피지컬
+혁신을 선도해 나가겠다
+고 말했다
+이 보도자료와 관련하여 보다 자세한 내용이나 취재를 원하시면 인공지능산업과 손창환 사무관
+(055-211-3972)
+이상훈 주무관
+(055-211-3973)
+에게 연락주시기 바랍니다
+경남도, 전국 최초 ‘피지컬AI 고속도로’ 구축 본격화 저작물은 공공누리 “출처표시+상업적이용금지” 조건에 따라 이용할 수 있습니다. 경남도, 국토지리정보원과 함께 개발제한구역 아날로그 항공사진 DB 구축 본격 추진
+경남자치경찰위, 여름 휴가철 맞아 ‘찾아가는 안심 지문등록’ 실시
+경상남도 민원 콜센터
+연락처 :
+055-120
+이 페이지에서 제공하는 정보에 대하여 만족하십니까? 매우만족
+불만족
+매우불만족
+의견 입력하기
+의견 등록하기
+0 / 100</t>
+        </is>
+      </c>
+      <c r="K45" s="2" t="inlineStr">
+        <is>
+          <t>정부부처·청·위원회</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:K1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -4881,7 +6153,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F23"/>
+  <dimension ref="A1:F24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -5406,6 +6678,28 @@
       </c>
       <c r="F23" t="n">
         <v>49.7</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>2026-07-21T15:17:48.738012+09:00</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>21</v>
+      </c>
+      <c r="C24" t="n">
+        <v>6</v>
+      </c>
+      <c r="D24" t="n">
+        <v>0</v>
+      </c>
+      <c r="E24" t="n">
+        <v>0</v>
+      </c>
+      <c r="F24" t="n">
+        <v>73.90000000000001</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
🤖 자동 수집: 2026-07-22 09:00 KST
</commit_message>
<xml_diff>
--- a/output/articles_daily.xlsx
+++ b/output/articles_daily.xlsx
@@ -4538,7 +4538,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F23"/>
+  <dimension ref="A1:F24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5055,6 +5055,28 @@
       </c>
       <c r="F23" t="n">
         <v>49.7</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>2026-07-22T09:00:31.045608+09:00</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>1</v>
+      </c>
+      <c r="C24" t="n">
+        <v>0</v>
+      </c>
+      <c r="D24" t="n">
+        <v>0</v>
+      </c>
+      <c r="E24" t="n">
+        <v>0</v>
+      </c>
+      <c r="F24" t="n">
+        <v>18.5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
🤖 자동 수집: 2026-07-23 09:08 KST
</commit_message>
<xml_diff>
--- a/output/articles_daily.xlsx
+++ b/output/articles_daily.xlsx
@@ -4538,7 +4538,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F24"/>
+  <dimension ref="A1:F25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5077,6 +5077,28 @@
       </c>
       <c r="F24" t="n">
         <v>18.5</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>2026-07-23T09:08:40.054630+09:00</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>0</v>
+      </c>
+      <c r="C25" t="n">
+        <v>0</v>
+      </c>
+      <c r="D25" t="n">
+        <v>0</v>
+      </c>
+      <c r="E25" t="n">
+        <v>0</v>
+      </c>
+      <c r="F25" t="n">
+        <v>15.7</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
🤖 자동 수집: 2026-07-27 09:08 KST
</commit_message>
<xml_diff>
--- a/output/articles_daily.xlsx
+++ b/output/articles_daily.xlsx
@@ -4538,7 +4538,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F25"/>
+  <dimension ref="A1:F26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5099,6 +5099,28 @@
       </c>
       <c r="F25" t="n">
         <v>15.7</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>2026-07-27T09:07:43.682617+09:00</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
+        <v>0</v>
+      </c>
+      <c r="C26" t="n">
+        <v>0</v>
+      </c>
+      <c r="D26" t="n">
+        <v>0</v>
+      </c>
+      <c r="E26" t="n">
+        <v>0</v>
+      </c>
+      <c r="F26" t="n">
+        <v>17.5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
🤖 자동 수집: 2026-07-28 09:08 KST
</commit_message>
<xml_diff>
--- a/output/articles_daily.xlsx
+++ b/output/articles_daily.xlsx
@@ -4538,7 +4538,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F26"/>
+  <dimension ref="A1:F27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5121,6 +5121,28 @@
       </c>
       <c r="F26" t="n">
         <v>17.5</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>2026-07-28T09:08:03.914504+09:00</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>0</v>
+      </c>
+      <c r="C27" t="n">
+        <v>0</v>
+      </c>
+      <c r="D27" t="n">
+        <v>0</v>
+      </c>
+      <c r="E27" t="n">
+        <v>0</v>
+      </c>
+      <c r="F27" t="n">
+        <v>14.7</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
🤖 자동 수집: 2026-07-29 09:05 KST
</commit_message>
<xml_diff>
--- a/output/articles_daily.xlsx
+++ b/output/articles_daily.xlsx
@@ -4538,7 +4538,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F27"/>
+  <dimension ref="A1:F28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5143,6 +5143,28 @@
       </c>
       <c r="F27" t="n">
         <v>14.7</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>2026-07-29T09:04:45.240041+09:00</t>
+        </is>
+      </c>
+      <c r="B28" t="n">
+        <v>0</v>
+      </c>
+      <c r="C28" t="n">
+        <v>0</v>
+      </c>
+      <c r="D28" t="n">
+        <v>0</v>
+      </c>
+      <c r="E28" t="n">
+        <v>0</v>
+      </c>
+      <c r="F28" t="n">
+        <v>15.6</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
🤖 자동 수집: 2026-07-30 09:05 KST
</commit_message>
<xml_diff>
--- a/output/articles_daily.xlsx
+++ b/output/articles_daily.xlsx
@@ -4538,7 +4538,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F28"/>
+  <dimension ref="A1:F29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5165,6 +5165,28 @@
       </c>
       <c r="F28" t="n">
         <v>15.6</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>2026-07-30T09:05:16.338981+09:00</t>
+        </is>
+      </c>
+      <c r="B29" t="n">
+        <v>0</v>
+      </c>
+      <c r="C29" t="n">
+        <v>0</v>
+      </c>
+      <c r="D29" t="n">
+        <v>0</v>
+      </c>
+      <c r="E29" t="n">
+        <v>0</v>
+      </c>
+      <c r="F29" t="n">
+        <v>16.3</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
🤖 자동 수집: 2026-07-31 09:10 KST
</commit_message>
<xml_diff>
--- a/output/articles_daily.xlsx
+++ b/output/articles_daily.xlsx
@@ -4538,7 +4538,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F29"/>
+  <dimension ref="A1:F30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5187,6 +5187,28 @@
       </c>
       <c r="F29" t="n">
         <v>16.3</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>2026-07-31T09:10:19.283932+09:00</t>
+        </is>
+      </c>
+      <c r="B30" t="n">
+        <v>0</v>
+      </c>
+      <c r="C30" t="n">
+        <v>0</v>
+      </c>
+      <c r="D30" t="n">
+        <v>0</v>
+      </c>
+      <c r="E30" t="n">
+        <v>0</v>
+      </c>
+      <c r="F30" t="n">
+        <v>14.9</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
🤖 자동 수집: 2026-08-01 09:07 KST
</commit_message>
<xml_diff>
--- a/output/articles_daily.xlsx
+++ b/output/articles_daily.xlsx
@@ -4538,7 +4538,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F30"/>
+  <dimension ref="A1:F31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5209,6 +5209,28 @@
       </c>
       <c r="F30" t="n">
         <v>14.9</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>2026-08-01T09:07:08.781604+09:00</t>
+        </is>
+      </c>
+      <c r="B31" t="n">
+        <v>0</v>
+      </c>
+      <c r="C31" t="n">
+        <v>0</v>
+      </c>
+      <c r="D31" t="n">
+        <v>0</v>
+      </c>
+      <c r="E31" t="n">
+        <v>0</v>
+      </c>
+      <c r="F31" t="n">
+        <v>15.4</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
🤖 자동 수집: 2026-08-03 09:04 KST
</commit_message>
<xml_diff>
--- a/output/articles_daily.xlsx
+++ b/output/articles_daily.xlsx
@@ -4538,7 +4538,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F31"/>
+  <dimension ref="A1:F32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5231,6 +5231,28 @@
       </c>
       <c r="F31" t="n">
         <v>15.4</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>2026-08-03T09:04:30.984454+09:00</t>
+        </is>
+      </c>
+      <c r="B32" t="n">
+        <v>0</v>
+      </c>
+      <c r="C32" t="n">
+        <v>0</v>
+      </c>
+      <c r="D32" t="n">
+        <v>0</v>
+      </c>
+      <c r="E32" t="n">
+        <v>0</v>
+      </c>
+      <c r="F32" t="n">
+        <v>17.3</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
🤖 자동 수집: 2026-08-04 09:13 KST
</commit_message>
<xml_diff>
--- a/output/articles_daily.xlsx
+++ b/output/articles_daily.xlsx
@@ -4538,7 +4538,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F32"/>
+  <dimension ref="A1:F33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5253,6 +5253,28 @@
       </c>
       <c r="F32" t="n">
         <v>17.3</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>2026-08-04T09:13:39.860856+09:00</t>
+        </is>
+      </c>
+      <c r="B33" t="n">
+        <v>0</v>
+      </c>
+      <c r="C33" t="n">
+        <v>0</v>
+      </c>
+      <c r="D33" t="n">
+        <v>0</v>
+      </c>
+      <c r="E33" t="n">
+        <v>0</v>
+      </c>
+      <c r="F33" t="n">
+        <v>16.1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
🤖 자동 수집: 2026-08-05 09:11 KST
</commit_message>
<xml_diff>
--- a/output/articles_daily.xlsx
+++ b/output/articles_daily.xlsx
@@ -4538,7 +4538,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F33"/>
+  <dimension ref="A1:F34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5274,6 +5274,28 @@
         <v>0</v>
       </c>
       <c r="F33" t="n">
+        <v>16.1</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>2026-08-05T09:11:08.171621+09:00</t>
+        </is>
+      </c>
+      <c r="B34" t="n">
+        <v>0</v>
+      </c>
+      <c r="C34" t="n">
+        <v>0</v>
+      </c>
+      <c r="D34" t="n">
+        <v>0</v>
+      </c>
+      <c r="E34" t="n">
+        <v>0</v>
+      </c>
+      <c r="F34" t="n">
         <v>16.1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
🤖 자동 수집: 2026-08-06 09:05 KST
</commit_message>
<xml_diff>
--- a/output/articles_daily.xlsx
+++ b/output/articles_daily.xlsx
@@ -4538,7 +4538,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F34"/>
+  <dimension ref="A1:F35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5297,6 +5297,28 @@
       </c>
       <c r="F34" t="n">
         <v>16.1</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>2026-08-06T09:05:29.667499+09:00</t>
+        </is>
+      </c>
+      <c r="B35" t="n">
+        <v>0</v>
+      </c>
+      <c r="C35" t="n">
+        <v>0</v>
+      </c>
+      <c r="D35" t="n">
+        <v>0</v>
+      </c>
+      <c r="E35" t="n">
+        <v>0</v>
+      </c>
+      <c r="F35" t="n">
+        <v>15.6</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
🤖 자동 수집: 2026-08-07 10:44 KST
</commit_message>
<xml_diff>
--- a/output/articles_daily.xlsx
+++ b/output/articles_daily.xlsx
@@ -4538,7 +4538,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F35"/>
+  <dimension ref="A1:F36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5319,6 +5319,28 @@
       </c>
       <c r="F35" t="n">
         <v>15.6</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>2026-08-07T10:43:47.250702+09:00</t>
+        </is>
+      </c>
+      <c r="B36" t="n">
+        <v>0</v>
+      </c>
+      <c r="C36" t="n">
+        <v>0</v>
+      </c>
+      <c r="D36" t="n">
+        <v>0</v>
+      </c>
+      <c r="E36" t="n">
+        <v>0</v>
+      </c>
+      <c r="F36" t="n">
+        <v>17.5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
🤖 자동 수집: 2026-08-10 08:38 KST
</commit_message>
<xml_diff>
--- a/output/articles_daily.xlsx
+++ b/output/articles_daily.xlsx
@@ -4538,7 +4538,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F36"/>
+  <dimension ref="A1:F37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5341,6 +5341,28 @@
       </c>
       <c r="F36" t="n">
         <v>17.5</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>2026-08-10T08:38:17.424407+09:00</t>
+        </is>
+      </c>
+      <c r="B37" t="n">
+        <v>0</v>
+      </c>
+      <c r="C37" t="n">
+        <v>0</v>
+      </c>
+      <c r="D37" t="n">
+        <v>0</v>
+      </c>
+      <c r="E37" t="n">
+        <v>0</v>
+      </c>
+      <c r="F37" t="n">
+        <v>14.5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
🤖 자동 수집: 2026-08-11 08:42 KST
</commit_message>
<xml_diff>
--- a/output/articles_daily.xlsx
+++ b/output/articles_daily.xlsx
@@ -4538,7 +4538,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F37"/>
+  <dimension ref="A1:F38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5362,6 +5362,28 @@
         <v>0</v>
       </c>
       <c r="F37" t="n">
+        <v>14.5</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>2026-08-11T08:42:12.129111+09:00</t>
+        </is>
+      </c>
+      <c r="B38" t="n">
+        <v>1</v>
+      </c>
+      <c r="C38" t="n">
+        <v>0</v>
+      </c>
+      <c r="D38" t="n">
+        <v>0</v>
+      </c>
+      <c r="E38" t="n">
+        <v>0</v>
+      </c>
+      <c r="F38" t="n">
         <v>14.5</v>
       </c>
     </row>

</xml_diff>

<commit_message>
🤖 자동 수집: 2026-08-12 08:51 KST
</commit_message>
<xml_diff>
--- a/output/articles_daily.xlsx
+++ b/output/articles_daily.xlsx
@@ -4538,7 +4538,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F38"/>
+  <dimension ref="A1:F39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5385,6 +5385,28 @@
       </c>
       <c r="F38" t="n">
         <v>14.5</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>2026-08-12T08:51:34.370189+09:00</t>
+        </is>
+      </c>
+      <c r="B39" t="n">
+        <v>0</v>
+      </c>
+      <c r="C39" t="n">
+        <v>0</v>
+      </c>
+      <c r="D39" t="n">
+        <v>0</v>
+      </c>
+      <c r="E39" t="n">
+        <v>0</v>
+      </c>
+      <c r="F39" t="n">
+        <v>15.7</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
🤖 자동 수집: 2026-08-13 08:51 KST
</commit_message>
<xml_diff>
--- a/output/articles_daily.xlsx
+++ b/output/articles_daily.xlsx
@@ -4538,7 +4538,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F39"/>
+  <dimension ref="A1:F40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5407,6 +5407,28 @@
       </c>
       <c r="F39" t="n">
         <v>15.7</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>2026-08-13T08:51:22.170812+09:00</t>
+        </is>
+      </c>
+      <c r="B40" t="n">
+        <v>0</v>
+      </c>
+      <c r="C40" t="n">
+        <v>0</v>
+      </c>
+      <c r="D40" t="n">
+        <v>0</v>
+      </c>
+      <c r="E40" t="n">
+        <v>0</v>
+      </c>
+      <c r="F40" t="n">
+        <v>15.8</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
🤖 자동 수집: 2026-08-14 08:51 KST
</commit_message>
<xml_diff>
--- a/output/articles_daily.xlsx
+++ b/output/articles_daily.xlsx
@@ -4538,7 +4538,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F40"/>
+  <dimension ref="A1:F41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5428,6 +5428,28 @@
         <v>0</v>
       </c>
       <c r="F40" t="n">
+        <v>15.8</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>2026-08-14T08:50:53.078059+09:00</t>
+        </is>
+      </c>
+      <c r="B41" t="n">
+        <v>1</v>
+      </c>
+      <c r="C41" t="n">
+        <v>0</v>
+      </c>
+      <c r="D41" t="n">
+        <v>0</v>
+      </c>
+      <c r="E41" t="n">
+        <v>0</v>
+      </c>
+      <c r="F41" t="n">
         <v>15.8</v>
       </c>
     </row>

</xml_diff>

<commit_message>
🤖 자동 수집: 2026-08-15 08:29 KST
</commit_message>
<xml_diff>
--- a/output/articles_daily.xlsx
+++ b/output/articles_daily.xlsx
@@ -4538,7 +4538,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F41"/>
+  <dimension ref="A1:F42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5451,6 +5451,28 @@
       </c>
       <c r="F41" t="n">
         <v>15.8</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>2026-08-15T08:29:08.219390+09:00</t>
+        </is>
+      </c>
+      <c r="B42" t="n">
+        <v>0</v>
+      </c>
+      <c r="C42" t="n">
+        <v>0</v>
+      </c>
+      <c r="D42" t="n">
+        <v>0</v>
+      </c>
+      <c r="E42" t="n">
+        <v>0</v>
+      </c>
+      <c r="F42" t="n">
+        <v>15.5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
🤖 자동 수집: 2026-08-16 08:27 KST
</commit_message>
<xml_diff>
--- a/output/articles_daily.xlsx
+++ b/output/articles_daily.xlsx
@@ -4538,7 +4538,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F42"/>
+  <dimension ref="A1:F43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5473,6 +5473,28 @@
       </c>
       <c r="F42" t="n">
         <v>15.5</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>2026-08-16T08:27:01.522620+09:00</t>
+        </is>
+      </c>
+      <c r="B43" t="n">
+        <v>0</v>
+      </c>
+      <c r="C43" t="n">
+        <v>0</v>
+      </c>
+      <c r="D43" t="n">
+        <v>0</v>
+      </c>
+      <c r="E43" t="n">
+        <v>0</v>
+      </c>
+      <c r="F43" t="n">
+        <v>17.9</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
🤖 자동 수집: 2026-08-17 08:27 KST
</commit_message>
<xml_diff>
--- a/output/articles_daily.xlsx
+++ b/output/articles_daily.xlsx
@@ -4538,7 +4538,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F43"/>
+  <dimension ref="A1:F44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5495,6 +5495,28 @@
       </c>
       <c r="F43" t="n">
         <v>17.9</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>2026-08-17T08:27:18.707332+09:00</t>
+        </is>
+      </c>
+      <c r="B44" t="n">
+        <v>0</v>
+      </c>
+      <c r="C44" t="n">
+        <v>0</v>
+      </c>
+      <c r="D44" t="n">
+        <v>0</v>
+      </c>
+      <c r="E44" t="n">
+        <v>0</v>
+      </c>
+      <c r="F44" t="n">
+        <v>15.9</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
🤖 자동 수집: 2026-08-18 08:30 KST
</commit_message>
<xml_diff>
--- a/output/articles_daily.xlsx
+++ b/output/articles_daily.xlsx
@@ -4538,7 +4538,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F44"/>
+  <dimension ref="A1:F45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5517,6 +5517,28 @@
       </c>
       <c r="F44" t="n">
         <v>15.9</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>2026-08-18T08:29:44.644877+09:00</t>
+        </is>
+      </c>
+      <c r="B45" t="n">
+        <v>1</v>
+      </c>
+      <c r="C45" t="n">
+        <v>0</v>
+      </c>
+      <c r="D45" t="n">
+        <v>0</v>
+      </c>
+      <c r="E45" t="n">
+        <v>0</v>
+      </c>
+      <c r="F45" t="n">
+        <v>14.8</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
🤖 자동 수집: 2026-08-19 08:28 KST
</commit_message>
<xml_diff>
--- a/output/articles_daily.xlsx
+++ b/output/articles_daily.xlsx
@@ -4538,7 +4538,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F45"/>
+  <dimension ref="A1:F46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5539,6 +5539,28 @@
       </c>
       <c r="F45" t="n">
         <v>14.8</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>2026-08-19T08:28:38.784822+09:00</t>
+        </is>
+      </c>
+      <c r="B46" t="n">
+        <v>0</v>
+      </c>
+      <c r="C46" t="n">
+        <v>0</v>
+      </c>
+      <c r="D46" t="n">
+        <v>0</v>
+      </c>
+      <c r="E46" t="n">
+        <v>0</v>
+      </c>
+      <c r="F46" t="n">
+        <v>16.1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
🤖 자동 수집: 2026-08-20 08:30 KST
</commit_message>
<xml_diff>
--- a/output/articles_daily.xlsx
+++ b/output/articles_daily.xlsx
@@ -4538,7 +4538,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F46"/>
+  <dimension ref="A1:F47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5561,6 +5561,28 @@
       </c>
       <c r="F46" t="n">
         <v>16.1</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>2026-08-20T08:30:17.225538+09:00</t>
+        </is>
+      </c>
+      <c r="B47" t="n">
+        <v>0</v>
+      </c>
+      <c r="C47" t="n">
+        <v>0</v>
+      </c>
+      <c r="D47" t="n">
+        <v>0</v>
+      </c>
+      <c r="E47" t="n">
+        <v>0</v>
+      </c>
+      <c r="F47" t="n">
+        <v>15.5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
🤖 자동 수집: 2026-08-22 08:31 KST
</commit_message>
<xml_diff>
--- a/output/articles_daily.xlsx
+++ b/output/articles_daily.xlsx
@@ -4538,7 +4538,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F47"/>
+  <dimension ref="A1:F48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5583,6 +5583,28 @@
       </c>
       <c r="F47" t="n">
         <v>15.5</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>2026-08-22T08:30:57.619702+09:00</t>
+        </is>
+      </c>
+      <c r="B48" t="n">
+        <v>0</v>
+      </c>
+      <c r="C48" t="n">
+        <v>0</v>
+      </c>
+      <c r="D48" t="n">
+        <v>0</v>
+      </c>
+      <c r="E48" t="n">
+        <v>0</v>
+      </c>
+      <c r="F48" t="n">
+        <v>16.2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
🤖 자동 수집: 2026-08-23 08:28 KST
</commit_message>
<xml_diff>
--- a/output/articles_daily.xlsx
+++ b/output/articles_daily.xlsx
@@ -4538,7 +4538,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F48"/>
+  <dimension ref="A1:F49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5605,6 +5605,28 @@
       </c>
       <c r="F48" t="n">
         <v>16.2</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>2026-08-23T08:28:13.646167+09:00</t>
+        </is>
+      </c>
+      <c r="B49" t="n">
+        <v>0</v>
+      </c>
+      <c r="C49" t="n">
+        <v>0</v>
+      </c>
+      <c r="D49" t="n">
+        <v>0</v>
+      </c>
+      <c r="E49" t="n">
+        <v>0</v>
+      </c>
+      <c r="F49" t="n">
+        <v>27.2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
🤖 자동 수집: 2026-08-24 08:28 KST
</commit_message>
<xml_diff>
--- a/output/articles_daily.xlsx
+++ b/output/articles_daily.xlsx
@@ -4538,7 +4538,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F49"/>
+  <dimension ref="A1:F50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5627,6 +5627,28 @@
       </c>
       <c r="F49" t="n">
         <v>27.2</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>2026-08-24T08:28:01.093790+09:00</t>
+        </is>
+      </c>
+      <c r="B50" t="n">
+        <v>0</v>
+      </c>
+      <c r="C50" t="n">
+        <v>0</v>
+      </c>
+      <c r="D50" t="n">
+        <v>0</v>
+      </c>
+      <c r="E50" t="n">
+        <v>0</v>
+      </c>
+      <c r="F50" t="n">
+        <v>15.7</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
🤖 자동 수집: 2026-08-25 08:28 KST
</commit_message>
<xml_diff>
--- a/output/articles_daily.xlsx
+++ b/output/articles_daily.xlsx
@@ -4538,7 +4538,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F50"/>
+  <dimension ref="A1:F51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5649,6 +5649,28 @@
       </c>
       <c r="F50" t="n">
         <v>15.7</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>2026-08-25T08:28:36.989692+09:00</t>
+        </is>
+      </c>
+      <c r="B51" t="n">
+        <v>0</v>
+      </c>
+      <c r="C51" t="n">
+        <v>0</v>
+      </c>
+      <c r="D51" t="n">
+        <v>0</v>
+      </c>
+      <c r="E51" t="n">
+        <v>0</v>
+      </c>
+      <c r="F51" t="n">
+        <v>15.5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
🤖 자동 수집: 2026-08-26 08:32 KST
</commit_message>
<xml_diff>
--- a/output/articles_daily.xlsx
+++ b/output/articles_daily.xlsx
@@ -4538,7 +4538,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F51"/>
+  <dimension ref="A1:F52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5671,6 +5671,28 @@
       </c>
       <c r="F51" t="n">
         <v>15.5</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>2026-08-26T08:32:27.491268+09:00</t>
+        </is>
+      </c>
+      <c r="B52" t="n">
+        <v>0</v>
+      </c>
+      <c r="C52" t="n">
+        <v>0</v>
+      </c>
+      <c r="D52" t="n">
+        <v>0</v>
+      </c>
+      <c r="E52" t="n">
+        <v>0</v>
+      </c>
+      <c r="F52" t="n">
+        <v>18</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
🤖 자동 수집: 2026-08-27 13:28 KST
</commit_message>
<xml_diff>
--- a/output/articles_daily.xlsx
+++ b/output/articles_daily.xlsx
@@ -4538,7 +4538,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F52"/>
+  <dimension ref="A1:F53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5693,6 +5693,28 @@
       </c>
       <c r="F52" t="n">
         <v>18</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>2026-08-27T13:28:25.609203+09:00</t>
+        </is>
+      </c>
+      <c r="B53" t="n">
+        <v>0</v>
+      </c>
+      <c r="C53" t="n">
+        <v>0</v>
+      </c>
+      <c r="D53" t="n">
+        <v>0</v>
+      </c>
+      <c r="E53" t="n">
+        <v>0</v>
+      </c>
+      <c r="F53" t="n">
+        <v>15.5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
🤖 자동 수집: 2026-08-28 15:52 KST
</commit_message>
<xml_diff>
--- a/output/articles_daily.xlsx
+++ b/output/articles_daily.xlsx
@@ -4538,7 +4538,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F53"/>
+  <dimension ref="A1:F54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5715,6 +5715,28 @@
       </c>
       <c r="F53" t="n">
         <v>15.5</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>2026-08-28T15:51:46.368681+09:00</t>
+        </is>
+      </c>
+      <c r="B54" t="n">
+        <v>0</v>
+      </c>
+      <c r="C54" t="n">
+        <v>0</v>
+      </c>
+      <c r="D54" t="n">
+        <v>0</v>
+      </c>
+      <c r="E54" t="n">
+        <v>0</v>
+      </c>
+      <c r="F54" t="n">
+        <v>16.4</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
🤖 자동 수집: 2026-08-29 13:07 KST
</commit_message>
<xml_diff>
--- a/output/articles_daily.xlsx
+++ b/output/articles_daily.xlsx
@@ -4538,7 +4538,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F54"/>
+  <dimension ref="A1:F55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5737,6 +5737,28 @@
       </c>
       <c r="F54" t="n">
         <v>16.4</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>2026-08-29T13:06:34.626391+09:00</t>
+        </is>
+      </c>
+      <c r="B55" t="n">
+        <v>0</v>
+      </c>
+      <c r="C55" t="n">
+        <v>0</v>
+      </c>
+      <c r="D55" t="n">
+        <v>0</v>
+      </c>
+      <c r="E55" t="n">
+        <v>0</v>
+      </c>
+      <c r="F55" t="n">
+        <v>26</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
🤖 자동 수집: 2026-08-30 10:12 KST
</commit_message>
<xml_diff>
--- a/output/articles_daily.xlsx
+++ b/output/articles_daily.xlsx
@@ -4538,7 +4538,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F55"/>
+  <dimension ref="A1:F56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5759,6 +5759,28 @@
       </c>
       <c r="F55" t="n">
         <v>26</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>2026-08-30T10:12:13.775029+09:00</t>
+        </is>
+      </c>
+      <c r="B56" t="n">
+        <v>0</v>
+      </c>
+      <c r="C56" t="n">
+        <v>0</v>
+      </c>
+      <c r="D56" t="n">
+        <v>0</v>
+      </c>
+      <c r="E56" t="n">
+        <v>0</v>
+      </c>
+      <c r="F56" t="n">
+        <v>15.5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
🤖 자동 수집: 2026-08-31 10:20 KST
</commit_message>
<xml_diff>
--- a/output/articles_daily.xlsx
+++ b/output/articles_daily.xlsx
@@ -4538,7 +4538,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F56"/>
+  <dimension ref="A1:F57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5781,6 +5781,28 @@
       </c>
       <c r="F56" t="n">
         <v>15.5</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>2026-08-31T10:19:44.290963+09:00</t>
+        </is>
+      </c>
+      <c r="B57" t="n">
+        <v>0</v>
+      </c>
+      <c r="C57" t="n">
+        <v>0</v>
+      </c>
+      <c r="D57" t="n">
+        <v>0</v>
+      </c>
+      <c r="E57" t="n">
+        <v>0</v>
+      </c>
+      <c r="F57" t="n">
+        <v>15.4</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
🤖 자동 수집: 2026-09-01 10:46 KST
</commit_message>
<xml_diff>
--- a/output/articles_daily.xlsx
+++ b/output/articles_daily.xlsx
@@ -4538,7 +4538,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F57"/>
+  <dimension ref="A1:F58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5803,6 +5803,28 @@
       </c>
       <c r="F57" t="n">
         <v>15.4</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>2026-09-01T10:45:48.632831+09:00</t>
+        </is>
+      </c>
+      <c r="B58" t="n">
+        <v>0</v>
+      </c>
+      <c r="C58" t="n">
+        <v>0</v>
+      </c>
+      <c r="D58" t="n">
+        <v>0</v>
+      </c>
+      <c r="E58" t="n">
+        <v>0</v>
+      </c>
+      <c r="F58" t="n">
+        <v>16.2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
🤖 자동 수집: 2026-09-02 09:58 KST
</commit_message>
<xml_diff>
--- a/output/articles_daily.xlsx
+++ b/output/articles_daily.xlsx
@@ -4538,7 +4538,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F58"/>
+  <dimension ref="A1:F59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5825,6 +5825,28 @@
       </c>
       <c r="F58" t="n">
         <v>16.2</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>2026-09-02T09:57:51.452830+09:00</t>
+        </is>
+      </c>
+      <c r="B59" t="n">
+        <v>0</v>
+      </c>
+      <c r="C59" t="n">
+        <v>0</v>
+      </c>
+      <c r="D59" t="n">
+        <v>0</v>
+      </c>
+      <c r="E59" t="n">
+        <v>0</v>
+      </c>
+      <c r="F59" t="n">
+        <v>15.2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
🤖 자동 수집: 2026-09-03 10:03 KST
</commit_message>
<xml_diff>
--- a/output/articles_daily.xlsx
+++ b/output/articles_daily.xlsx
@@ -4538,7 +4538,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F59"/>
+  <dimension ref="A1:F60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5847,6 +5847,28 @@
       </c>
       <c r="F59" t="n">
         <v>15.2</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>2026-09-03T10:03:09.409669+09:00</t>
+        </is>
+      </c>
+      <c r="B60" t="n">
+        <v>0</v>
+      </c>
+      <c r="C60" t="n">
+        <v>0</v>
+      </c>
+      <c r="D60" t="n">
+        <v>0</v>
+      </c>
+      <c r="E60" t="n">
+        <v>0</v>
+      </c>
+      <c r="F60" t="n">
+        <v>14.8</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
🤖 자동 수집: 2026-09-04 09:54 KST
</commit_message>
<xml_diff>
--- a/output/articles_daily.xlsx
+++ b/output/articles_daily.xlsx
@@ -4538,7 +4538,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F60"/>
+  <dimension ref="A1:F61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5869,6 +5869,28 @@
       </c>
       <c r="F60" t="n">
         <v>14.8</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>2026-09-04T09:54:29.440482+09:00</t>
+        </is>
+      </c>
+      <c r="B61" t="n">
+        <v>0</v>
+      </c>
+      <c r="C61" t="n">
+        <v>0</v>
+      </c>
+      <c r="D61" t="n">
+        <v>0</v>
+      </c>
+      <c r="E61" t="n">
+        <v>0</v>
+      </c>
+      <c r="F61" t="n">
+        <v>15.4</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
🤖 자동 수집: 2026-09-05 09:48 KST
</commit_message>
<xml_diff>
--- a/output/articles_daily.xlsx
+++ b/output/articles_daily.xlsx
@@ -4538,7 +4538,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F61"/>
+  <dimension ref="A1:F62"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5891,6 +5891,28 @@
       </c>
       <c r="F61" t="n">
         <v>15.4</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>2026-09-05T09:48:36.906578+09:00</t>
+        </is>
+      </c>
+      <c r="B62" t="n">
+        <v>0</v>
+      </c>
+      <c r="C62" t="n">
+        <v>0</v>
+      </c>
+      <c r="D62" t="n">
+        <v>0</v>
+      </c>
+      <c r="E62" t="n">
+        <v>0</v>
+      </c>
+      <c r="F62" t="n">
+        <v>15.6</v>
       </c>
     </row>
   </sheetData>

</xml_diff>